<commit_message>
driver data - 2000
</commit_message>
<xml_diff>
--- a/Data_Files/Driver_Experience.xlsx
+++ b/Data_Files/Driver_Experience.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimonOM\Repositories\Formula-1-Constructor-Repository\Data_Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFCF17F8-9A94-4DD9-8AD7-5B5DF04802D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21409134-6BD0-4CA6-8AA5-0F5A7316DD90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-12660" windowWidth="16440" windowHeight="28320" xr2:uid="{3A639250-557D-4B08-A9B4-7BAD64B6336B}"/>
+    <workbookView xWindow="28695" yWindow="-12540" windowWidth="16410" windowHeight="14145" xr2:uid="{3A639250-557D-4B08-A9B4-7BAD64B6336B}"/>
   </bookViews>
   <sheets>
     <sheet name="Driver_Lineup_Experience" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="153">
   <si>
     <t>Driver</t>
   </si>
@@ -1725,6 +1725,9 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
+      <c r="AC2">
+        <v>17</v>
+      </c>
       <c r="AD2">
         <v>9</v>
       </c>
@@ -1750,13 +1753,16 @@
         <v>16</v>
       </c>
       <c r="AL2">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
+      <c r="AC3">
+        <v>17</v>
+      </c>
       <c r="AD3">
         <v>16</v>
       </c>
@@ -1789,7 +1795,9 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="AC4" s="1"/>
+      <c r="AC4" s="1">
+        <v>0</v>
+      </c>
       <c r="AD4" s="1">
         <v>0</v>
       </c>
@@ -1822,6 +1830,9 @@
       <c r="A5" t="s">
         <v>4</v>
       </c>
+      <c r="AC5">
+        <v>17</v>
+      </c>
       <c r="AD5">
         <v>16</v>
       </c>
@@ -1854,7 +1865,9 @@
       <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="AC6" s="1"/>
+      <c r="AC6" s="1">
+        <v>0</v>
+      </c>
       <c r="AD6" s="1">
         <v>0</v>
       </c>
@@ -1887,6 +1900,9 @@
       <c r="A7" t="s">
         <v>6</v>
       </c>
+      <c r="AC7">
+        <v>17</v>
+      </c>
       <c r="AD7">
         <v>16</v>
       </c>
@@ -1920,7 +1936,9 @@
         <v>7</v>
       </c>
       <c r="AB8" s="1"/>
-      <c r="AC8" s="1"/>
+      <c r="AC8" s="1">
+        <v>0</v>
+      </c>
       <c r="AD8" s="1">
         <v>0</v>
       </c>
@@ -1953,6 +1971,9 @@
       <c r="A9" t="s">
         <v>8</v>
       </c>
+      <c r="AC9">
+        <v>16</v>
+      </c>
       <c r="AD9" s="1">
         <v>0</v>
       </c>
@@ -1985,6 +2006,9 @@
       <c r="A10" t="s">
         <v>9</v>
       </c>
+      <c r="AC10">
+        <v>17</v>
+      </c>
       <c r="AD10">
         <v>16</v>
       </c>
@@ -2017,6 +2041,9 @@
       <c r="A11" t="s">
         <v>10</v>
       </c>
+      <c r="AC11" s="1">
+        <v>0</v>
+      </c>
       <c r="AD11">
         <v>16</v>
       </c>
@@ -2049,6 +2076,9 @@
       <c r="A12" t="s">
         <v>11</v>
       </c>
+      <c r="AC12">
+        <v>17</v>
+      </c>
       <c r="AD12" s="1">
         <v>0</v>
       </c>
@@ -2081,6 +2111,9 @@
       <c r="A13" t="s">
         <v>12</v>
       </c>
+      <c r="AC13">
+        <v>17</v>
+      </c>
       <c r="AD13">
         <v>16</v>
       </c>
@@ -2114,7 +2147,9 @@
         <v>13</v>
       </c>
       <c r="AB14" s="1"/>
-      <c r="AC14" s="1"/>
+      <c r="AC14" s="1">
+        <v>0</v>
+      </c>
       <c r="AD14" s="1">
         <v>0</v>
       </c>
@@ -2147,6 +2182,9 @@
       <c r="A15" t="s">
         <v>14</v>
       </c>
+      <c r="AC15">
+        <v>17</v>
+      </c>
       <c r="AD15">
         <v>16</v>
       </c>
@@ -2179,6 +2217,9 @@
       <c r="A16" t="s">
         <v>15</v>
       </c>
+      <c r="AC16">
+        <v>16</v>
+      </c>
       <c r="AD16">
         <v>16</v>
       </c>
@@ -2211,6 +2252,9 @@
       <c r="A17" t="s">
         <v>16</v>
       </c>
+      <c r="AC17">
+        <v>16</v>
+      </c>
       <c r="AD17">
         <v>16</v>
       </c>
@@ -2244,7 +2288,9 @@
         <v>17</v>
       </c>
       <c r="AB18" s="1"/>
-      <c r="AC18" s="1"/>
+      <c r="AC18" s="1">
+        <v>0</v>
+      </c>
       <c r="AD18" s="1">
         <v>0</v>
       </c>
@@ -2278,7 +2324,9 @@
         <v>85</v>
       </c>
       <c r="AB19" s="1"/>
-      <c r="AC19" s="1"/>
+      <c r="AC19" s="1">
+        <v>0</v>
+      </c>
       <c r="AD19" s="1">
         <v>0</v>
       </c>
@@ -2311,7 +2359,9 @@
       <c r="A20" t="s">
         <v>18</v>
       </c>
-      <c r="AC20" s="1"/>
+      <c r="AC20" s="1">
+        <v>0</v>
+      </c>
       <c r="AD20" s="1">
         <v>0</v>
       </c>
@@ -2344,7 +2394,9 @@
       <c r="A21" t="s">
         <v>19</v>
       </c>
-      <c r="AC21" s="1"/>
+      <c r="AC21" s="1">
+        <v>0</v>
+      </c>
       <c r="AD21" s="1">
         <v>0</v>
       </c>
@@ -2377,6 +2429,9 @@
       <c r="A22" t="s">
         <v>55</v>
       </c>
+      <c r="AC22">
+        <v>17</v>
+      </c>
       <c r="AD22">
         <v>16</v>
       </c>
@@ -2409,6 +2464,9 @@
       <c r="A23" t="s">
         <v>21</v>
       </c>
+      <c r="AC23">
+        <v>15</v>
+      </c>
       <c r="AD23">
         <v>9</v>
       </c>
@@ -2442,7 +2500,9 @@
         <v>22</v>
       </c>
       <c r="AB24" s="1"/>
-      <c r="AC24" s="1"/>
+      <c r="AC24" s="1">
+        <v>0</v>
+      </c>
       <c r="AD24" s="1">
         <v>0</v>
       </c>
@@ -2475,7 +2535,9 @@
       <c r="A25" t="s">
         <v>44</v>
       </c>
-      <c r="AC25" s="1"/>
+      <c r="AC25" s="1">
+        <v>0</v>
+      </c>
       <c r="AD25" s="1">
         <v>0</v>
       </c>
@@ -2510,7 +2572,9 @@
       </c>
       <c r="AA26" s="1"/>
       <c r="AB26" s="1"/>
-      <c r="AC26" s="1"/>
+      <c r="AC26" s="1">
+        <v>0</v>
+      </c>
       <c r="AD26" s="1">
         <v>0</v>
       </c>
@@ -2545,7 +2609,9 @@
       </c>
       <c r="AA27" s="1"/>
       <c r="AB27" s="1"/>
-      <c r="AC27" s="1"/>
+      <c r="AC27" s="1">
+        <v>0</v>
+      </c>
       <c r="AD27" s="1">
         <v>0</v>
       </c>
@@ -2578,6 +2644,9 @@
       <c r="A28" t="s">
         <v>47</v>
       </c>
+      <c r="AC28">
+        <v>17</v>
+      </c>
       <c r="AD28" s="1">
         <v>0</v>
       </c>
@@ -2612,7 +2681,9 @@
       </c>
       <c r="AA29" s="1"/>
       <c r="AB29" s="1"/>
-      <c r="AC29" s="1"/>
+      <c r="AC29" s="1">
+        <v>0</v>
+      </c>
       <c r="AD29" s="1">
         <v>0</v>
       </c>
@@ -2647,7 +2718,9 @@
       </c>
       <c r="AA30" s="1"/>
       <c r="AB30" s="1"/>
-      <c r="AC30" s="1"/>
+      <c r="AC30" s="1">
+        <v>0</v>
+      </c>
       <c r="AD30" s="1">
         <v>0</v>
       </c>
@@ -2680,7 +2753,9 @@
       <c r="A31" t="s">
         <v>54</v>
       </c>
-      <c r="AC31" s="1"/>
+      <c r="AC31" s="1">
+        <v>0</v>
+      </c>
       <c r="AD31" s="1">
         <v>0</v>
       </c>
@@ -2715,7 +2790,9 @@
       </c>
       <c r="AA32" s="1"/>
       <c r="AB32" s="1"/>
-      <c r="AC32" s="1"/>
+      <c r="AC32" s="1">
+        <v>0</v>
+      </c>
       <c r="AD32" s="1">
         <v>0</v>
       </c>
@@ -2748,6 +2825,9 @@
       <c r="A33" t="s">
         <v>53</v>
       </c>
+      <c r="AC33">
+        <v>17</v>
+      </c>
       <c r="AD33">
         <v>16</v>
       </c>
@@ -2782,7 +2862,9 @@
       </c>
       <c r="AA34" s="1"/>
       <c r="AB34" s="1"/>
-      <c r="AC34" s="1"/>
+      <c r="AC34" s="1">
+        <v>0</v>
+      </c>
       <c r="AD34" s="1">
         <v>0</v>
       </c>
@@ -2817,7 +2899,9 @@
       </c>
       <c r="AA35" s="1"/>
       <c r="AB35" s="1"/>
-      <c r="AC35" s="1"/>
+      <c r="AC35" s="1">
+        <v>0</v>
+      </c>
       <c r="AD35" s="1">
         <v>0</v>
       </c>
@@ -2852,7 +2936,9 @@
       </c>
       <c r="AA36" s="1"/>
       <c r="AB36" s="1"/>
-      <c r="AC36" s="1"/>
+      <c r="AC36" s="1">
+        <v>0</v>
+      </c>
       <c r="AD36" s="1">
         <v>0</v>
       </c>
@@ -2887,7 +2973,9 @@
       </c>
       <c r="AA37" s="1"/>
       <c r="AB37" s="1"/>
-      <c r="AC37" s="1"/>
+      <c r="AC37" s="1">
+        <v>0</v>
+      </c>
       <c r="AD37" s="1">
         <v>0</v>
       </c>
@@ -2922,7 +3010,9 @@
       </c>
       <c r="AA38" s="1"/>
       <c r="AB38" s="1"/>
-      <c r="AC38" s="1"/>
+      <c r="AC38" s="1">
+        <v>0</v>
+      </c>
       <c r="AD38" s="1">
         <v>0</v>
       </c>
@@ -2958,7 +3048,9 @@
       <c r="Z39" s="1"/>
       <c r="AA39" s="1"/>
       <c r="AB39" s="1"/>
-      <c r="AC39" s="1"/>
+      <c r="AC39" s="1">
+        <v>0</v>
+      </c>
       <c r="AD39" s="1">
         <v>0</v>
       </c>
@@ -2994,7 +3086,9 @@
       <c r="Z40" s="1"/>
       <c r="AA40" s="1"/>
       <c r="AB40" s="1"/>
-      <c r="AC40" s="1"/>
+      <c r="AC40" s="1">
+        <v>0</v>
+      </c>
       <c r="AD40" s="1">
         <v>0</v>
       </c>
@@ -3027,6 +3121,9 @@
       <c r="A41" t="s">
         <v>64</v>
       </c>
+      <c r="AC41">
+        <v>17</v>
+      </c>
       <c r="AD41">
         <v>12</v>
       </c>
@@ -3062,7 +3159,9 @@
       <c r="Z42" s="1"/>
       <c r="AA42" s="1"/>
       <c r="AB42" s="1"/>
-      <c r="AC42" s="1"/>
+      <c r="AC42" s="1">
+        <v>0</v>
+      </c>
       <c r="AD42" s="1">
         <v>0</v>
       </c>
@@ -3098,7 +3197,9 @@
       <c r="Z43" s="1"/>
       <c r="AA43" s="1"/>
       <c r="AB43" s="1"/>
-      <c r="AC43" s="1"/>
+      <c r="AC43" s="1">
+        <v>0</v>
+      </c>
       <c r="AD43" s="1">
         <v>0</v>
       </c>
@@ -3135,7 +3236,9 @@
       <c r="Z44" s="1"/>
       <c r="AA44" s="1"/>
       <c r="AB44" s="1"/>
-      <c r="AC44" s="1"/>
+      <c r="AC44" s="1">
+        <v>0</v>
+      </c>
       <c r="AD44" s="1">
         <v>0</v>
       </c>
@@ -3167,6 +3270,9 @@
     <row r="45" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>68</v>
+      </c>
+      <c r="AC45">
+        <v>17</v>
       </c>
       <c r="AD45">
         <v>16</v>
@@ -3204,7 +3310,9 @@
       <c r="Z46" s="1"/>
       <c r="AA46" s="1"/>
       <c r="AB46" s="1"/>
-      <c r="AC46" s="1"/>
+      <c r="AC46" s="1">
+        <v>0</v>
+      </c>
       <c r="AD46" s="1">
         <v>0</v>
       </c>
@@ -3241,7 +3349,9 @@
       <c r="Z47" s="1"/>
       <c r="AA47" s="1"/>
       <c r="AB47" s="1"/>
-      <c r="AC47" s="1"/>
+      <c r="AC47" s="1">
+        <v>0</v>
+      </c>
       <c r="AD47" s="1">
         <v>0</v>
       </c>
@@ -3278,7 +3388,9 @@
       <c r="Z48" s="1"/>
       <c r="AA48" s="1"/>
       <c r="AB48" s="1"/>
-      <c r="AC48" s="1"/>
+      <c r="AC48" s="1">
+        <v>0</v>
+      </c>
       <c r="AD48" s="1">
         <v>0</v>
       </c>
@@ -3315,7 +3427,9 @@
       <c r="Z49" s="1"/>
       <c r="AA49" s="1"/>
       <c r="AB49" s="1"/>
-      <c r="AC49" s="1"/>
+      <c r="AC49" s="1">
+        <v>0</v>
+      </c>
       <c r="AD49" s="1">
         <v>0</v>
       </c>
@@ -3352,7 +3466,9 @@
       <c r="Z50" s="1"/>
       <c r="AA50" s="1"/>
       <c r="AB50" s="1"/>
-      <c r="AC50" s="1"/>
+      <c r="AC50" s="1">
+        <v>0</v>
+      </c>
       <c r="AD50" s="1">
         <v>0</v>
       </c>
@@ -3390,7 +3506,9 @@
       <c r="Z51" s="1"/>
       <c r="AA51" s="1"/>
       <c r="AB51" s="1"/>
-      <c r="AC51" s="1"/>
+      <c r="AC51" s="1">
+        <v>0</v>
+      </c>
       <c r="AD51" s="1">
         <v>0</v>
       </c>
@@ -3428,7 +3546,9 @@
       <c r="Z52" s="1"/>
       <c r="AA52" s="1"/>
       <c r="AB52" s="1"/>
-      <c r="AC52" s="1"/>
+      <c r="AC52" s="1">
+        <v>0</v>
+      </c>
       <c r="AD52" s="1">
         <v>0</v>
       </c>
@@ -3466,7 +3586,9 @@
       <c r="Z53" s="1"/>
       <c r="AA53" s="1"/>
       <c r="AB53" s="1"/>
-      <c r="AC53" s="1"/>
+      <c r="AC53" s="1">
+        <v>0</v>
+      </c>
       <c r="AD53" s="1">
         <v>0</v>
       </c>
@@ -3504,7 +3626,9 @@
       <c r="Z54" s="1"/>
       <c r="AA54" s="1"/>
       <c r="AB54" s="1"/>
-      <c r="AC54" s="1"/>
+      <c r="AC54" s="1">
+        <v>0</v>
+      </c>
       <c r="AD54" s="1">
         <v>0</v>
       </c>
@@ -3542,7 +3666,9 @@
       <c r="Z55" s="1"/>
       <c r="AA55" s="1"/>
       <c r="AB55" s="1"/>
-      <c r="AC55" s="1"/>
+      <c r="AC55" s="1">
+        <v>0</v>
+      </c>
       <c r="AD55" s="1">
         <v>0</v>
       </c>
@@ -3580,7 +3706,9 @@
       <c r="Z56" s="1"/>
       <c r="AA56" s="1"/>
       <c r="AB56" s="1"/>
-      <c r="AC56" s="1"/>
+      <c r="AC56" s="1">
+        <v>0</v>
+      </c>
       <c r="AD56" s="1">
         <v>0</v>
       </c>
@@ -3619,7 +3747,9 @@
       <c r="Z57" s="1"/>
       <c r="AA57" s="1"/>
       <c r="AB57" s="1"/>
-      <c r="AC57" s="1"/>
+      <c r="AC57" s="1">
+        <v>0</v>
+      </c>
       <c r="AD57" s="1">
         <v>0</v>
       </c>
@@ -3658,7 +3788,9 @@
       <c r="Z58" s="1"/>
       <c r="AA58" s="1"/>
       <c r="AB58" s="1"/>
-      <c r="AC58" s="1"/>
+      <c r="AC58" s="1">
+        <v>0</v>
+      </c>
       <c r="AD58" s="1">
         <v>0</v>
       </c>
@@ -3697,7 +3829,9 @@
       <c r="Z59" s="1"/>
       <c r="AA59" s="1"/>
       <c r="AB59" s="1"/>
-      <c r="AC59" s="1"/>
+      <c r="AC59" s="1">
+        <v>0</v>
+      </c>
       <c r="AD59" s="1">
         <v>0</v>
       </c>
@@ -3736,7 +3870,9 @@
       <c r="Z60" s="1"/>
       <c r="AA60" s="1"/>
       <c r="AB60" s="1"/>
-      <c r="AC60" s="1"/>
+      <c r="AC60" s="1">
+        <v>0</v>
+      </c>
       <c r="AD60" s="1">
         <v>0</v>
       </c>
@@ -3775,7 +3911,9 @@
       <c r="Z61" s="1"/>
       <c r="AA61" s="1"/>
       <c r="AB61" s="1"/>
-      <c r="AC61" s="1"/>
+      <c r="AC61" s="1">
+        <v>0</v>
+      </c>
       <c r="AD61" s="1">
         <v>0</v>
       </c>
@@ -3815,7 +3953,9 @@
       <c r="Z62" s="1"/>
       <c r="AA62" s="1"/>
       <c r="AB62" s="1"/>
-      <c r="AC62" s="1"/>
+      <c r="AC62" s="1">
+        <v>0</v>
+      </c>
       <c r="AD62" s="1">
         <v>0</v>
       </c>
@@ -3855,7 +3995,9 @@
       <c r="Z63" s="1"/>
       <c r="AA63" s="1"/>
       <c r="AB63" s="1"/>
-      <c r="AC63" s="1"/>
+      <c r="AC63" s="1">
+        <v>0</v>
+      </c>
       <c r="AD63" s="1">
         <v>0</v>
       </c>
@@ -3896,7 +4038,9 @@
       <c r="Z64" s="1"/>
       <c r="AA64" s="1"/>
       <c r="AB64" s="1"/>
-      <c r="AC64" s="1"/>
+      <c r="AC64" s="1">
+        <v>0</v>
+      </c>
       <c r="AD64" s="1">
         <v>0</v>
       </c>
@@ -3937,7 +4081,9 @@
       <c r="Z65" s="1"/>
       <c r="AA65" s="1"/>
       <c r="AB65" s="1"/>
-      <c r="AC65" s="1"/>
+      <c r="AC65" s="1">
+        <v>0</v>
+      </c>
       <c r="AD65" s="1">
         <v>0</v>
       </c>
@@ -3978,7 +4124,9 @@
       <c r="Z66" s="1"/>
       <c r="AA66" s="1"/>
       <c r="AB66" s="1"/>
-      <c r="AC66" s="1"/>
+      <c r="AC66" s="1">
+        <v>0</v>
+      </c>
       <c r="AD66" s="1">
         <v>0</v>
       </c>
@@ -4019,7 +4167,9 @@
       <c r="Z67" s="1"/>
       <c r="AA67" s="1"/>
       <c r="AB67" s="1"/>
-      <c r="AC67" s="1"/>
+      <c r="AC67" s="1">
+        <v>0</v>
+      </c>
       <c r="AD67" s="1">
         <v>0</v>
       </c>
@@ -4051,6 +4201,33 @@
     <row r="68" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>92</v>
+      </c>
+      <c r="U68" s="1">
+        <v>0</v>
+      </c>
+      <c r="V68" s="1">
+        <v>0</v>
+      </c>
+      <c r="W68" s="1">
+        <v>0</v>
+      </c>
+      <c r="X68" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y68" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z68" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA68" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB68" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC68" s="1">
+        <v>0</v>
       </c>
       <c r="AD68">
         <v>15</v>
@@ -4093,7 +4270,9 @@
       <c r="Z69" s="1"/>
       <c r="AA69" s="1"/>
       <c r="AB69" s="1"/>
-      <c r="AC69" s="1"/>
+      <c r="AC69" s="1">
+        <v>0</v>
+      </c>
       <c r="AD69" s="1">
         <v>0</v>
       </c>
@@ -4135,7 +4314,9 @@
       <c r="Z70" s="1"/>
       <c r="AA70" s="1"/>
       <c r="AB70" s="1"/>
-      <c r="AC70" s="1"/>
+      <c r="AC70" s="1">
+        <v>0</v>
+      </c>
       <c r="AD70" s="1">
         <v>0</v>
       </c>
@@ -4177,7 +4358,9 @@
       <c r="Z71" s="1"/>
       <c r="AA71" s="1"/>
       <c r="AB71" s="1"/>
-      <c r="AC71" s="1"/>
+      <c r="AC71" s="1">
+        <v>0</v>
+      </c>
       <c r="AD71" s="1">
         <v>0</v>
       </c>
@@ -4219,7 +4402,9 @@
       <c r="Z72" s="1"/>
       <c r="AA72" s="1"/>
       <c r="AB72" s="1"/>
-      <c r="AC72" s="1"/>
+      <c r="AC72" s="1">
+        <v>0</v>
+      </c>
       <c r="AD72" s="1">
         <v>0</v>
       </c>
@@ -4261,7 +4446,9 @@
       <c r="Z73" s="1"/>
       <c r="AA73" s="1"/>
       <c r="AB73" s="1"/>
-      <c r="AC73" s="1"/>
+      <c r="AC73" s="1">
+        <v>0</v>
+      </c>
       <c r="AD73" s="1">
         <v>0</v>
       </c>
@@ -4304,7 +4491,9 @@
       <c r="Z74" s="1"/>
       <c r="AA74" s="1"/>
       <c r="AB74" s="1"/>
-      <c r="AC74" s="1"/>
+      <c r="AC74" s="1">
+        <v>0</v>
+      </c>
       <c r="AD74" s="1">
         <v>0</v>
       </c>
@@ -4347,7 +4536,9 @@
       <c r="Z75" s="1"/>
       <c r="AA75" s="1"/>
       <c r="AB75" s="1"/>
-      <c r="AC75" s="1"/>
+      <c r="AC75" s="1">
+        <v>0</v>
+      </c>
       <c r="AD75" s="1">
         <v>0</v>
       </c>
@@ -4390,7 +4581,9 @@
       <c r="Z76" s="1"/>
       <c r="AA76" s="1"/>
       <c r="AB76" s="1"/>
-      <c r="AC76" s="1"/>
+      <c r="AC76" s="1">
+        <v>0</v>
+      </c>
       <c r="AD76" s="1">
         <v>0</v>
       </c>
@@ -4433,7 +4626,9 @@
       <c r="Z77" s="1"/>
       <c r="AA77" s="1"/>
       <c r="AB77" s="1"/>
-      <c r="AC77" s="1"/>
+      <c r="AC77" s="1">
+        <v>0</v>
+      </c>
       <c r="AD77" s="1">
         <v>0</v>
       </c>
@@ -4476,7 +4671,9 @@
       <c r="Z78" s="1"/>
       <c r="AA78" s="1"/>
       <c r="AB78" s="1"/>
-      <c r="AC78" s="1"/>
+      <c r="AC78" s="1">
+        <v>0</v>
+      </c>
       <c r="AD78" s="1">
         <v>0</v>
       </c>
@@ -4520,7 +4717,9 @@
       <c r="Z79" s="1"/>
       <c r="AA79" s="1"/>
       <c r="AB79" s="1"/>
-      <c r="AC79" s="1"/>
+      <c r="AC79" s="1">
+        <v>0</v>
+      </c>
       <c r="AD79" s="1">
         <v>0</v>
       </c>
@@ -4564,7 +4763,9 @@
       <c r="Z80" s="1"/>
       <c r="AA80" s="1"/>
       <c r="AB80" s="1"/>
-      <c r="AC80" s="1"/>
+      <c r="AC80" s="1">
+        <v>0</v>
+      </c>
       <c r="AD80" s="1">
         <v>0</v>
       </c>
@@ -4609,7 +4810,9 @@
       <c r="Z81" s="1"/>
       <c r="AA81" s="1"/>
       <c r="AB81" s="1"/>
-      <c r="AC81" s="1"/>
+      <c r="AC81" s="1">
+        <v>0</v>
+      </c>
       <c r="AD81" s="1">
         <v>0</v>
       </c>
@@ -4654,7 +4857,9 @@
       <c r="Z82" s="1"/>
       <c r="AA82" s="1"/>
       <c r="AB82" s="1"/>
-      <c r="AC82" s="1"/>
+      <c r="AC82" s="1">
+        <v>0</v>
+      </c>
       <c r="AD82" s="1">
         <v>0</v>
       </c>
@@ -4699,7 +4904,9 @@
       <c r="Z83" s="1"/>
       <c r="AA83" s="1"/>
       <c r="AB83" s="1"/>
-      <c r="AC83" s="1"/>
+      <c r="AC83" s="1">
+        <v>0</v>
+      </c>
       <c r="AD83" s="1">
         <v>0</v>
       </c>
@@ -4744,7 +4951,9 @@
       <c r="Z84" s="1"/>
       <c r="AA84" s="1"/>
       <c r="AB84" s="1"/>
-      <c r="AC84" s="1"/>
+      <c r="AC84" s="1">
+        <v>0</v>
+      </c>
       <c r="AD84" s="1">
         <v>0</v>
       </c>
@@ -4789,7 +4998,9 @@
       <c r="Z85" s="1"/>
       <c r="AA85" s="1"/>
       <c r="AB85" s="1"/>
-      <c r="AC85" s="1"/>
+      <c r="AC85" s="1">
+        <v>0</v>
+      </c>
       <c r="AD85" s="1">
         <v>0</v>
       </c>
@@ -4835,7 +5046,9 @@
       <c r="Z86" s="1"/>
       <c r="AA86" s="1"/>
       <c r="AB86" s="1"/>
-      <c r="AC86" s="1"/>
+      <c r="AC86" s="1">
+        <v>0</v>
+      </c>
       <c r="AD86" s="1">
         <v>0</v>
       </c>
@@ -4881,7 +5094,9 @@
       <c r="Z87" s="1"/>
       <c r="AA87" s="1"/>
       <c r="AB87" s="1"/>
-      <c r="AC87" s="1"/>
+      <c r="AC87" s="1">
+        <v>0</v>
+      </c>
       <c r="AD87" s="1">
         <v>0</v>
       </c>
@@ -4927,7 +5142,9 @@
       <c r="Z88" s="1"/>
       <c r="AA88" s="1"/>
       <c r="AB88" s="1"/>
-      <c r="AC88" s="1"/>
+      <c r="AC88" s="1">
+        <v>0</v>
+      </c>
       <c r="AD88" s="1">
         <v>0</v>
       </c>
@@ -4973,7 +5190,9 @@
       <c r="Z89" s="1"/>
       <c r="AA89" s="1"/>
       <c r="AB89" s="1"/>
-      <c r="AC89" s="1"/>
+      <c r="AC89" s="1">
+        <v>0</v>
+      </c>
       <c r="AD89" s="1">
         <v>0</v>
       </c>
@@ -5020,7 +5239,9 @@
       <c r="Z90" s="1"/>
       <c r="AA90" s="1"/>
       <c r="AB90" s="1"/>
-      <c r="AC90" s="1"/>
+      <c r="AC90" s="1">
+        <v>0</v>
+      </c>
       <c r="AD90" s="1">
         <v>0</v>
       </c>
@@ -5067,7 +5288,9 @@
       <c r="Z91" s="1"/>
       <c r="AA91" s="1"/>
       <c r="AB91" s="1"/>
-      <c r="AC91" s="1"/>
+      <c r="AC91" s="1">
+        <v>0</v>
+      </c>
       <c r="AD91" s="1">
         <v>0</v>
       </c>
@@ -5114,7 +5337,9 @@
       <c r="Z92" s="1"/>
       <c r="AA92" s="1"/>
       <c r="AB92" s="1"/>
-      <c r="AC92" s="1"/>
+      <c r="AC92" s="1">
+        <v>0</v>
+      </c>
       <c r="AD92" s="1">
         <v>0</v>
       </c>
@@ -5161,7 +5386,9 @@
       <c r="Z93" s="1"/>
       <c r="AA93" s="1"/>
       <c r="AB93" s="1"/>
-      <c r="AC93" s="1"/>
+      <c r="AC93" s="1">
+        <v>0</v>
+      </c>
       <c r="AD93" s="1">
         <v>0</v>
       </c>
@@ -5208,7 +5435,9 @@
       <c r="Z94" s="1"/>
       <c r="AA94" s="1"/>
       <c r="AB94" s="1"/>
-      <c r="AC94" s="1"/>
+      <c r="AC94" s="1">
+        <v>0</v>
+      </c>
       <c r="AD94" s="1">
         <v>0</v>
       </c>
@@ -5256,7 +5485,9 @@
       <c r="Z95" s="1"/>
       <c r="AA95" s="1"/>
       <c r="AB95" s="1"/>
-      <c r="AC95" s="1"/>
+      <c r="AC95" s="1">
+        <v>0</v>
+      </c>
       <c r="AD95" s="1">
         <v>0</v>
       </c>
@@ -5304,7 +5535,9 @@
       <c r="Z96" s="1"/>
       <c r="AA96" s="1"/>
       <c r="AB96" s="1"/>
-      <c r="AC96" s="1"/>
+      <c r="AC96" s="1">
+        <v>0</v>
+      </c>
       <c r="AD96" s="1">
         <v>0</v>
       </c>
@@ -5352,7 +5585,9 @@
       <c r="Z97" s="1"/>
       <c r="AA97" s="1"/>
       <c r="AB97" s="1"/>
-      <c r="AC97" s="1"/>
+      <c r="AC97" s="1">
+        <v>0</v>
+      </c>
       <c r="AD97" s="1">
         <v>0</v>
       </c>
@@ -5400,7 +5635,9 @@
       <c r="Z98" s="1"/>
       <c r="AA98" s="1"/>
       <c r="AB98" s="1"/>
-      <c r="AC98" s="1"/>
+      <c r="AC98" s="1">
+        <v>0</v>
+      </c>
       <c r="AD98" s="1">
         <v>0</v>
       </c>
@@ -5448,7 +5685,9 @@
       <c r="Z99" s="1"/>
       <c r="AA99" s="1"/>
       <c r="AB99" s="1"/>
-      <c r="AC99" s="1"/>
+      <c r="AC99" s="1">
+        <v>0</v>
+      </c>
       <c r="AD99" s="1">
         <v>0</v>
       </c>
@@ -5497,7 +5736,9 @@
       <c r="Z100" s="1"/>
       <c r="AA100" s="1"/>
       <c r="AB100" s="1"/>
-      <c r="AC100" s="1"/>
+      <c r="AC100" s="1">
+        <v>0</v>
+      </c>
       <c r="AD100" s="1">
         <v>0</v>
       </c>
@@ -5546,7 +5787,9 @@
       <c r="Z101" s="1"/>
       <c r="AA101" s="1"/>
       <c r="AB101" s="1"/>
-      <c r="AC101" s="1"/>
+      <c r="AC101" s="1">
+        <v>0</v>
+      </c>
       <c r="AD101" s="1">
         <v>0</v>
       </c>
@@ -5595,7 +5838,9 @@
       <c r="Z102" s="1"/>
       <c r="AA102" s="1"/>
       <c r="AB102" s="1"/>
-      <c r="AC102" s="1"/>
+      <c r="AC102" s="1">
+        <v>0</v>
+      </c>
       <c r="AD102" s="1">
         <v>0</v>
       </c>
@@ -5644,7 +5889,9 @@
       <c r="Z103" s="1"/>
       <c r="AA103" s="1"/>
       <c r="AB103" s="1"/>
-      <c r="AC103" s="1"/>
+      <c r="AC103" s="1">
+        <v>0</v>
+      </c>
       <c r="AD103" s="1">
         <v>0</v>
       </c>
@@ -5694,7 +5941,9 @@
       <c r="Z104" s="1"/>
       <c r="AA104" s="1"/>
       <c r="AB104" s="1"/>
-      <c r="AC104" s="1"/>
+      <c r="AC104" s="1">
+        <v>0</v>
+      </c>
       <c r="AD104" s="1">
         <v>0</v>
       </c>
@@ -5744,7 +5993,9 @@
       <c r="Z105" s="1"/>
       <c r="AA105" s="1"/>
       <c r="AB105" s="1"/>
-      <c r="AC105" s="1"/>
+      <c r="AC105" s="1">
+        <v>0</v>
+      </c>
       <c r="AD105" s="1">
         <v>0</v>
       </c>
@@ -5795,7 +6046,9 @@
       <c r="Z106" s="1"/>
       <c r="AA106" s="1"/>
       <c r="AB106" s="1"/>
-      <c r="AC106" s="1"/>
+      <c r="AC106" s="1">
+        <v>0</v>
+      </c>
       <c r="AD106" s="1">
         <v>0</v>
       </c>
@@ -5846,7 +6099,9 @@
       <c r="Z107" s="1"/>
       <c r="AA107" s="1"/>
       <c r="AB107" s="1"/>
-      <c r="AC107" s="1"/>
+      <c r="AC107" s="1">
+        <v>0</v>
+      </c>
       <c r="AD107" s="1">
         <v>0</v>
       </c>
@@ -5897,7 +6152,9 @@
       <c r="Z108" s="1"/>
       <c r="AA108" s="1"/>
       <c r="AB108" s="1"/>
-      <c r="AC108" s="1"/>
+      <c r="AC108" s="1">
+        <v>0</v>
+      </c>
       <c r="AD108" s="1">
         <v>0</v>
       </c>
@@ -5949,7 +6206,9 @@
       <c r="Z109" s="1"/>
       <c r="AA109" s="1"/>
       <c r="AB109" s="1"/>
-      <c r="AC109" s="1"/>
+      <c r="AC109" s="1">
+        <v>0</v>
+      </c>
       <c r="AD109" s="1">
         <v>0</v>
       </c>
@@ -6001,7 +6260,9 @@
       <c r="Z110" s="1"/>
       <c r="AA110" s="1"/>
       <c r="AB110" s="1"/>
-      <c r="AC110" s="1"/>
+      <c r="AC110" s="1">
+        <v>0</v>
+      </c>
       <c r="AD110" s="1">
         <v>0</v>
       </c>
@@ -6053,7 +6314,9 @@
       <c r="Z111" s="1"/>
       <c r="AA111" s="1"/>
       <c r="AB111" s="1"/>
-      <c r="AC111" s="1"/>
+      <c r="AC111" s="1">
+        <v>0</v>
+      </c>
       <c r="AD111" s="1">
         <v>0</v>
       </c>
@@ -6106,7 +6369,9 @@
       <c r="Z112" s="1"/>
       <c r="AA112" s="1"/>
       <c r="AB112" s="1"/>
-      <c r="AC112" s="1"/>
+      <c r="AC112" s="1">
+        <v>0</v>
+      </c>
       <c r="AD112" s="1">
         <v>0</v>
       </c>
@@ -6159,7 +6424,9 @@
       <c r="Z113" s="1"/>
       <c r="AA113" s="1"/>
       <c r="AB113" s="1"/>
-      <c r="AC113" s="1"/>
+      <c r="AC113" s="1">
+        <v>0</v>
+      </c>
       <c r="AD113" s="1">
         <v>0</v>
       </c>
@@ -6212,7 +6479,9 @@
       <c r="Z114" s="1"/>
       <c r="AA114" s="1"/>
       <c r="AB114" s="1"/>
-      <c r="AC114" s="1"/>
+      <c r="AC114" s="1">
+        <v>0</v>
+      </c>
       <c r="AD114" s="1">
         <v>0</v>
       </c>
@@ -6266,7 +6535,9 @@
       <c r="Z115" s="1"/>
       <c r="AA115" s="1"/>
       <c r="AB115" s="1"/>
-      <c r="AC115" s="1"/>
+      <c r="AC115" s="1">
+        <v>0</v>
+      </c>
       <c r="AD115" s="1">
         <v>0</v>
       </c>
@@ -6320,7 +6591,9 @@
       <c r="Z116" s="1"/>
       <c r="AA116" s="1"/>
       <c r="AB116" s="1"/>
-      <c r="AC116" s="1"/>
+      <c r="AC116" s="1">
+        <v>0</v>
+      </c>
       <c r="AD116" s="1">
         <v>0</v>
       </c>
@@ -6375,7 +6648,9 @@
       <c r="Z117" s="1"/>
       <c r="AA117" s="1"/>
       <c r="AB117" s="1"/>
-      <c r="AC117" s="1"/>
+      <c r="AC117" s="1">
+        <v>0</v>
+      </c>
       <c r="AD117" s="1">
         <v>0</v>
       </c>
@@ -6430,7 +6705,9 @@
       <c r="Z118" s="1"/>
       <c r="AA118" s="1"/>
       <c r="AB118" s="1"/>
-      <c r="AC118" s="1"/>
+      <c r="AC118" s="1">
+        <v>0</v>
+      </c>
       <c r="AD118" s="1">
         <v>0</v>
       </c>
@@ -6485,7 +6762,9 @@
       <c r="Z119" s="1"/>
       <c r="AA119" s="1"/>
       <c r="AB119" s="1"/>
-      <c r="AC119" s="1"/>
+      <c r="AC119" s="1">
+        <v>0</v>
+      </c>
       <c r="AD119" s="1">
         <v>0</v>
       </c>
@@ -6541,7 +6820,9 @@
       <c r="Z120" s="1"/>
       <c r="AA120" s="1"/>
       <c r="AB120" s="1"/>
-      <c r="AC120" s="1"/>
+      <c r="AC120" s="1">
+        <v>0</v>
+      </c>
       <c r="AD120" s="1">
         <v>0</v>
       </c>
@@ -6597,7 +6878,9 @@
       <c r="Z121" s="1"/>
       <c r="AA121" s="1"/>
       <c r="AB121" s="1"/>
-      <c r="AC121" s="1"/>
+      <c r="AC121" s="1">
+        <v>0</v>
+      </c>
       <c r="AD121" s="1">
         <v>0</v>
       </c>
@@ -6653,7 +6936,9 @@
       <c r="Z122" s="1"/>
       <c r="AA122" s="1"/>
       <c r="AB122" s="1"/>
-      <c r="AC122" s="1"/>
+      <c r="AC122" s="1">
+        <v>0</v>
+      </c>
       <c r="AD122" s="1">
         <v>0</v>
       </c>
@@ -6710,7 +6995,9 @@
       <c r="Z123" s="1"/>
       <c r="AA123" s="1"/>
       <c r="AB123" s="1"/>
-      <c r="AC123" s="1"/>
+      <c r="AC123" s="1">
+        <v>0</v>
+      </c>
       <c r="AD123" s="1">
         <v>0</v>
       </c>
@@ -6767,7 +7054,9 @@
       <c r="Z124" s="1"/>
       <c r="AA124" s="1"/>
       <c r="AB124" s="1"/>
-      <c r="AC124" s="1"/>
+      <c r="AC124" s="1">
+        <v>0</v>
+      </c>
       <c r="AD124" s="1">
         <v>0</v>
       </c>
@@ -6824,7 +7113,9 @@
       <c r="Z125" s="1"/>
       <c r="AA125" s="1"/>
       <c r="AB125" s="1"/>
-      <c r="AC125" s="1"/>
+      <c r="AC125" s="1">
+        <v>0</v>
+      </c>
       <c r="AD125" s="1">
         <v>0</v>
       </c>
@@ -6882,7 +7173,9 @@
       <c r="Z126" s="1"/>
       <c r="AA126" s="1"/>
       <c r="AB126" s="1"/>
-      <c r="AC126" s="1"/>
+      <c r="AC126" s="1">
+        <v>0</v>
+      </c>
       <c r="AD126" s="1">
         <v>0</v>
       </c>
@@ -7914,12 +8207,1107 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFC06B72-571E-40C4-AD69-3294909EA05A}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:S18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.85546875" customWidth="1"/>
+    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I1" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N1" t="s">
+        <v>36</v>
+      </c>
+      <c r="O1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P1" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>39</v>
+      </c>
+      <c r="R1" t="s">
+        <v>40</v>
+      </c>
+      <c r="S1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <f>SUM(C2:S2)</f>
+        <v>17</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2">
+        <v>1</v>
+      </c>
+      <c r="O2">
+        <v>1</v>
+      </c>
+      <c r="P2">
+        <v>1</v>
+      </c>
+      <c r="Q2">
+        <v>1</v>
+      </c>
+      <c r="R2">
+        <v>1</v>
+      </c>
+      <c r="S2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <f t="shared" ref="B3:B18" si="0">SUM(C3:S3)</f>
+        <v>17</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+      <c r="N3">
+        <v>1</v>
+      </c>
+      <c r="O3">
+        <v>1</v>
+      </c>
+      <c r="P3">
+        <v>1</v>
+      </c>
+      <c r="Q3">
+        <v>1</v>
+      </c>
+      <c r="R3">
+        <v>1</v>
+      </c>
+      <c r="S3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+      <c r="N4">
+        <v>1</v>
+      </c>
+      <c r="O4">
+        <v>1</v>
+      </c>
+      <c r="P4">
+        <v>1</v>
+      </c>
+      <c r="Q4">
+        <v>1</v>
+      </c>
+      <c r="R4">
+        <v>1</v>
+      </c>
+      <c r="S4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+      <c r="N5">
+        <v>1</v>
+      </c>
+      <c r="O5">
+        <v>1</v>
+      </c>
+      <c r="P5">
+        <v>1</v>
+      </c>
+      <c r="Q5">
+        <v>1</v>
+      </c>
+      <c r="R5">
+        <v>1</v>
+      </c>
+      <c r="S5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+      <c r="N6">
+        <v>1</v>
+      </c>
+      <c r="O6">
+        <v>1</v>
+      </c>
+      <c r="P6">
+        <v>1</v>
+      </c>
+      <c r="Q6">
+        <v>1</v>
+      </c>
+      <c r="R6">
+        <v>1</v>
+      </c>
+      <c r="S6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
+      <c r="N7">
+        <v>1</v>
+      </c>
+      <c r="O7">
+        <v>1</v>
+      </c>
+      <c r="P7">
+        <v>1</v>
+      </c>
+      <c r="Q7">
+        <v>1</v>
+      </c>
+      <c r="R7">
+        <v>1</v>
+      </c>
+      <c r="S7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8">
+        <v>1</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8">
+        <v>1</v>
+      </c>
+      <c r="N8">
+        <v>1</v>
+      </c>
+      <c r="O8">
+        <v>1</v>
+      </c>
+      <c r="P8">
+        <v>1</v>
+      </c>
+      <c r="Q8">
+        <v>1</v>
+      </c>
+      <c r="R8">
+        <v>1</v>
+      </c>
+      <c r="S8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9">
+        <v>1</v>
+      </c>
+      <c r="N9">
+        <v>1</v>
+      </c>
+      <c r="O9">
+        <v>1</v>
+      </c>
+      <c r="P9">
+        <v>1</v>
+      </c>
+      <c r="Q9">
+        <v>1</v>
+      </c>
+      <c r="R9">
+        <v>1</v>
+      </c>
+      <c r="S9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10">
+        <v>1</v>
+      </c>
+      <c r="N10">
+        <v>1</v>
+      </c>
+      <c r="O10">
+        <v>1</v>
+      </c>
+      <c r="P10">
+        <v>1</v>
+      </c>
+      <c r="Q10">
+        <v>1</v>
+      </c>
+      <c r="R10">
+        <v>1</v>
+      </c>
+      <c r="S10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11">
+        <v>1</v>
+      </c>
+      <c r="N11">
+        <v>1</v>
+      </c>
+      <c r="O11">
+        <v>1</v>
+      </c>
+      <c r="P11">
+        <v>1</v>
+      </c>
+      <c r="Q11">
+        <v>1</v>
+      </c>
+      <c r="R11">
+        <v>1</v>
+      </c>
+      <c r="S11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <v>1</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
+      <c r="K12">
+        <v>1</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>1</v>
+      </c>
+      <c r="N12">
+        <v>1</v>
+      </c>
+      <c r="O12">
+        <v>1</v>
+      </c>
+      <c r="P12">
+        <v>1</v>
+      </c>
+      <c r="Q12">
+        <v>1</v>
+      </c>
+      <c r="R12">
+        <v>1</v>
+      </c>
+      <c r="S12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>1</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="J13">
+        <v>1</v>
+      </c>
+      <c r="K13">
+        <v>1</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13">
+        <v>1</v>
+      </c>
+      <c r="N13">
+        <v>1</v>
+      </c>
+      <c r="O13">
+        <v>1</v>
+      </c>
+      <c r="P13">
+        <v>1</v>
+      </c>
+      <c r="Q13">
+        <v>1</v>
+      </c>
+      <c r="R13">
+        <v>1</v>
+      </c>
+      <c r="S13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <v>1</v>
+      </c>
+      <c r="J14">
+        <v>1</v>
+      </c>
+      <c r="K14">
+        <v>1</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14">
+        <v>1</v>
+      </c>
+      <c r="N14">
+        <v>1</v>
+      </c>
+      <c r="O14">
+        <v>1</v>
+      </c>
+      <c r="P14">
+        <v>1</v>
+      </c>
+      <c r="Q14">
+        <v>1</v>
+      </c>
+      <c r="R14">
+        <v>1</v>
+      </c>
+      <c r="S14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
+      <c r="K15">
+        <v>1</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15">
+        <v>1</v>
+      </c>
+      <c r="N15">
+        <v>1</v>
+      </c>
+      <c r="O15">
+        <v>1</v>
+      </c>
+      <c r="P15">
+        <v>1</v>
+      </c>
+      <c r="Q15">
+        <v>1</v>
+      </c>
+      <c r="R15">
+        <v>1</v>
+      </c>
+      <c r="S15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16">
+        <v>1</v>
+      </c>
+      <c r="J16">
+        <v>1</v>
+      </c>
+      <c r="K16">
+        <v>1</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16">
+        <v>1</v>
+      </c>
+      <c r="N16">
+        <v>1</v>
+      </c>
+      <c r="O16">
+        <v>1</v>
+      </c>
+      <c r="P16">
+        <v>1</v>
+      </c>
+      <c r="Q16">
+        <v>1</v>
+      </c>
+      <c r="R16">
+        <v>1</v>
+      </c>
+      <c r="S16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>1</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+      <c r="J17">
+        <v>1</v>
+      </c>
+      <c r="K17">
+        <v>1</v>
+      </c>
+      <c r="L17">
+        <v>1</v>
+      </c>
+      <c r="M17">
+        <v>1</v>
+      </c>
+      <c r="N17">
+        <v>1</v>
+      </c>
+      <c r="O17">
+        <v>1</v>
+      </c>
+      <c r="P17">
+        <v>1</v>
+      </c>
+      <c r="Q17">
+        <v>1</v>
+      </c>
+      <c r="R17">
+        <v>1</v>
+      </c>
+      <c r="S17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>1</v>
+      </c>
+      <c r="I18">
+        <v>1</v>
+      </c>
+      <c r="J18">
+        <v>1</v>
+      </c>
+      <c r="K18">
+        <v>1</v>
+      </c>
+      <c r="L18">
+        <v>1</v>
+      </c>
+      <c r="M18">
+        <v>1</v>
+      </c>
+      <c r="N18">
+        <v>1</v>
+      </c>
+      <c r="O18">
+        <v>1</v>
+      </c>
+      <c r="P18">
+        <v>1</v>
+      </c>
+      <c r="Q18">
+        <v>1</v>
+      </c>
+      <c r="R18">
+        <v>1</v>
+      </c>
+      <c r="S18">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -9153,7 +10541,7 @@
       </c>
       <c r="B2">
         <f>SUM(C2:R2)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -9186,7 +10574,7 @@
         <v>0</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N2">
         <v>1</v>

</xml_diff>

<commit_message>
driver data - 2002, 2003
</commit_message>
<xml_diff>
--- a/Data_Files/Driver_Experience.xlsx
+++ b/Data_Files/Driver_Experience.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimonOM\Repositories\Formula-1-Constructor-Repository\Data_Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF884681-884A-4F04-A19D-4184EF2DF36D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB09F56D-2401-4DF1-8D83-BC50326EE30E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="-12540" windowWidth="16410" windowHeight="14145" xr2:uid="{3A639250-557D-4B08-A9B4-7BAD64B6336B}"/>
+    <workbookView xWindow="28695" yWindow="-12540" windowWidth="16410" windowHeight="14145" firstSheet="6" activeTab="13" xr2:uid="{3A639250-557D-4B08-A9B4-7BAD64B6336B}"/>
   </bookViews>
   <sheets>
     <sheet name="Driver_Lineup_Experience" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1069" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1085" uniqueCount="153">
   <si>
     <t>Driver</t>
   </si>
@@ -1725,6 +1725,12 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
+      <c r="Z2">
+        <v>16</v>
+      </c>
+      <c r="AA2">
+        <v>17</v>
+      </c>
       <c r="AB2">
         <v>17</v>
       </c>
@@ -1763,6 +1769,12 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
+      <c r="Z3">
+        <v>16</v>
+      </c>
+      <c r="AA3">
+        <v>16</v>
+      </c>
       <c r="AB3">
         <v>17</v>
       </c>
@@ -1801,6 +1813,12 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
+      <c r="Z4">
+        <v>16</v>
+      </c>
+      <c r="AA4">
+        <v>17</v>
+      </c>
       <c r="AB4">
         <v>16</v>
       </c>
@@ -1839,6 +1857,12 @@
       <c r="A5" t="s">
         <v>4</v>
       </c>
+      <c r="Z5">
+        <v>16</v>
+      </c>
+      <c r="AA5">
+        <v>17</v>
+      </c>
       <c r="AB5">
         <v>17</v>
       </c>
@@ -1877,6 +1901,12 @@
       <c r="A6" t="s">
         <v>5</v>
       </c>
+      <c r="Z6">
+        <v>16</v>
+      </c>
+      <c r="AA6">
+        <v>17</v>
+      </c>
       <c r="AB6">
         <v>17</v>
       </c>
@@ -1915,6 +1945,12 @@
       <c r="A7" t="s">
         <v>6</v>
       </c>
+      <c r="Z7">
+        <v>15</v>
+      </c>
+      <c r="AA7">
+        <v>17</v>
+      </c>
       <c r="AB7">
         <v>17</v>
       </c>
@@ -1953,6 +1989,9 @@
       <c r="A8" t="s">
         <v>7</v>
       </c>
+      <c r="AA8">
+        <v>16</v>
+      </c>
       <c r="AB8" s="1">
         <v>0</v>
       </c>
@@ -1991,6 +2030,9 @@
       <c r="A9" t="s">
         <v>8</v>
       </c>
+      <c r="AA9">
+        <v>17</v>
+      </c>
       <c r="AB9">
         <v>17</v>
       </c>
@@ -2029,6 +2071,9 @@
       <c r="A10" t="s">
         <v>9</v>
       </c>
+      <c r="AA10">
+        <v>17</v>
+      </c>
       <c r="AB10">
         <v>17</v>
       </c>
@@ -2067,6 +2112,9 @@
       <c r="A11" t="s">
         <v>10</v>
       </c>
+      <c r="AA11">
+        <v>17</v>
+      </c>
       <c r="AB11">
         <v>17</v>
       </c>
@@ -2105,6 +2153,12 @@
       <c r="A12" t="s">
         <v>11</v>
       </c>
+      <c r="Z12">
+        <v>15</v>
+      </c>
+      <c r="AA12">
+        <v>17</v>
+      </c>
       <c r="AB12">
         <v>17</v>
       </c>
@@ -2143,6 +2197,12 @@
       <c r="A13" t="s">
         <v>12</v>
       </c>
+      <c r="Z13">
+        <v>16</v>
+      </c>
+      <c r="AA13">
+        <v>17</v>
+      </c>
       <c r="AB13">
         <v>17</v>
       </c>
@@ -2181,6 +2241,9 @@
       <c r="A14" t="s">
         <v>13</v>
       </c>
+      <c r="AA14">
+        <v>17</v>
+      </c>
       <c r="AB14" s="1">
         <v>0</v>
       </c>
@@ -2219,6 +2282,12 @@
       <c r="A15" t="s">
         <v>14</v>
       </c>
+      <c r="Z15">
+        <v>16</v>
+      </c>
+      <c r="AA15">
+        <v>16</v>
+      </c>
       <c r="AB15">
         <v>17</v>
       </c>
@@ -2257,6 +2326,9 @@
       <c r="A16" t="s">
         <v>15</v>
       </c>
+      <c r="AA16">
+        <v>17</v>
+      </c>
       <c r="AB16">
         <v>13</v>
       </c>
@@ -2295,6 +2367,9 @@
       <c r="A17" t="s">
         <v>16</v>
       </c>
+      <c r="AA17">
+        <v>17</v>
+      </c>
       <c r="AB17">
         <v>16</v>
       </c>
@@ -2333,6 +2408,12 @@
       <c r="A18" t="s">
         <v>17</v>
       </c>
+      <c r="Z18">
+        <v>16</v>
+      </c>
+      <c r="AA18">
+        <v>16</v>
+      </c>
       <c r="AB18" s="1">
         <v>0</v>
       </c>
@@ -2371,6 +2452,9 @@
       <c r="A19" t="s">
         <v>85</v>
       </c>
+      <c r="AA19">
+        <v>2</v>
+      </c>
       <c r="AB19" s="1">
         <v>0</v>
       </c>
@@ -2409,6 +2493,9 @@
       <c r="A20" t="s">
         <v>18</v>
       </c>
+      <c r="AA20">
+        <v>11</v>
+      </c>
       <c r="AB20">
         <v>3</v>
       </c>
@@ -2447,6 +2534,9 @@
       <c r="A21" t="s">
         <v>19</v>
       </c>
+      <c r="AA21">
+        <v>10</v>
+      </c>
       <c r="AB21">
         <v>17</v>
       </c>
@@ -2485,6 +2575,12 @@
       <c r="A22" t="s">
         <v>55</v>
       </c>
+      <c r="Z22">
+        <v>15</v>
+      </c>
+      <c r="AA22">
+        <v>11</v>
+      </c>
       <c r="AB22">
         <v>15</v>
       </c>
@@ -2523,6 +2619,9 @@
       <c r="A23" t="s">
         <v>21</v>
       </c>
+      <c r="AA23">
+        <v>17</v>
+      </c>
       <c r="AB23">
         <v>0</v>
       </c>
@@ -2561,6 +2660,9 @@
       <c r="A24" t="s">
         <v>22</v>
       </c>
+      <c r="AA24">
+        <v>16</v>
+      </c>
       <c r="AB24" s="1">
         <v>0</v>
       </c>
@@ -2599,6 +2701,12 @@
       <c r="A25" t="s">
         <v>44</v>
       </c>
+      <c r="Z25">
+        <v>16</v>
+      </c>
+      <c r="AA25">
+        <v>0</v>
+      </c>
       <c r="AB25">
         <v>16</v>
       </c>
@@ -2637,7 +2745,9 @@
       <c r="A26" t="s">
         <v>45</v>
       </c>
-      <c r="AA26" s="1"/>
+      <c r="AA26" s="1">
+        <v>0</v>
+      </c>
       <c r="AB26" s="1">
         <v>0</v>
       </c>
@@ -2676,7 +2786,9 @@
       <c r="A27" t="s">
         <v>46</v>
       </c>
-      <c r="AA27" s="1"/>
+      <c r="AA27" s="1">
+        <v>0</v>
+      </c>
       <c r="AB27" s="1">
         <v>0</v>
       </c>
@@ -2715,6 +2827,9 @@
       <c r="A28" t="s">
         <v>47</v>
       </c>
+      <c r="AA28">
+        <v>0</v>
+      </c>
       <c r="AB28">
         <v>17</v>
       </c>
@@ -2753,7 +2868,9 @@
       <c r="A29" t="s">
         <v>48</v>
       </c>
-      <c r="AA29" s="1"/>
+      <c r="AA29" s="1">
+        <v>0</v>
+      </c>
       <c r="AB29" s="1">
         <v>0</v>
       </c>
@@ -2792,7 +2909,12 @@
       <c r="A30" t="s">
         <v>49</v>
       </c>
-      <c r="AA30" s="1"/>
+      <c r="Z30">
+        <v>16</v>
+      </c>
+      <c r="AA30" s="1">
+        <v>0</v>
+      </c>
       <c r="AB30" s="1">
         <v>0</v>
       </c>
@@ -2831,6 +2953,9 @@
       <c r="A31" t="s">
         <v>53</v>
       </c>
+      <c r="AA31">
+        <v>0</v>
+      </c>
       <c r="AB31">
         <v>0</v>
       </c>
@@ -2869,7 +2994,9 @@
       <c r="A32" t="s">
         <v>57</v>
       </c>
-      <c r="AA32" s="1"/>
+      <c r="AA32" s="1">
+        <v>0</v>
+      </c>
       <c r="AB32" s="1">
         <v>0</v>
       </c>
@@ -2908,7 +3035,9 @@
       <c r="A33" t="s">
         <v>58</v>
       </c>
-      <c r="AA33" s="1"/>
+      <c r="AA33" s="1">
+        <v>0</v>
+      </c>
       <c r="AB33" s="1">
         <v>0</v>
       </c>
@@ -2947,7 +3076,9 @@
       <c r="A34" t="s">
         <v>59</v>
       </c>
-      <c r="AA34" s="1"/>
+      <c r="AA34" s="1">
+        <v>0</v>
+      </c>
       <c r="AB34" s="1">
         <v>0</v>
       </c>
@@ -2986,7 +3117,9 @@
       <c r="A35" t="s">
         <v>60</v>
       </c>
-      <c r="AA35" s="1"/>
+      <c r="AA35" s="1">
+        <v>0</v>
+      </c>
       <c r="AB35" s="1">
         <v>0</v>
       </c>
@@ -3025,7 +3158,9 @@
       <c r="A36" t="s">
         <v>61</v>
       </c>
-      <c r="AA36" s="1"/>
+      <c r="AA36" s="1">
+        <v>0</v>
+      </c>
       <c r="AB36" s="1">
         <v>0</v>
       </c>
@@ -3065,7 +3200,9 @@
         <v>62</v>
       </c>
       <c r="Z37" s="1"/>
-      <c r="AA37" s="1"/>
+      <c r="AA37" s="1">
+        <v>0</v>
+      </c>
       <c r="AB37" s="1">
         <v>0</v>
       </c>
@@ -3105,7 +3242,9 @@
         <v>63</v>
       </c>
       <c r="Z38" s="1"/>
-      <c r="AA38" s="1"/>
+      <c r="AA38" s="1">
+        <v>0</v>
+      </c>
       <c r="AB38" s="1">
         <v>0</v>
       </c>
@@ -3144,6 +3283,9 @@
       <c r="A39" t="s">
         <v>64</v>
       </c>
+      <c r="AA39">
+        <v>0</v>
+      </c>
       <c r="AB39">
         <v>2</v>
       </c>
@@ -3183,7 +3325,9 @@
         <v>65</v>
       </c>
       <c r="Z40" s="1"/>
-      <c r="AA40" s="1"/>
+      <c r="AA40" s="1">
+        <v>0</v>
+      </c>
       <c r="AB40" s="1">
         <v>0</v>
       </c>
@@ -3223,7 +3367,9 @@
         <v>66</v>
       </c>
       <c r="Z41" s="1"/>
-      <c r="AA41" s="1"/>
+      <c r="AA41" s="1">
+        <v>0</v>
+      </c>
       <c r="AB41" s="1">
         <v>0</v>
       </c>
@@ -3264,7 +3410,9 @@
       </c>
       <c r="Y42" s="1"/>
       <c r="Z42" s="1"/>
-      <c r="AA42" s="1"/>
+      <c r="AA42" s="1">
+        <v>0</v>
+      </c>
       <c r="AB42" s="1">
         <v>0</v>
       </c>
@@ -3303,6 +3451,9 @@
       <c r="A43" t="s">
         <v>68</v>
       </c>
+      <c r="AA43">
+        <v>0</v>
+      </c>
       <c r="AB43">
         <v>0</v>
       </c>
@@ -3343,7 +3494,9 @@
       </c>
       <c r="Y44" s="1"/>
       <c r="Z44" s="1"/>
-      <c r="AA44" s="1"/>
+      <c r="AA44" s="1">
+        <v>0</v>
+      </c>
       <c r="AB44" s="1">
         <v>0</v>
       </c>
@@ -3384,7 +3537,9 @@
       </c>
       <c r="Y45" s="1"/>
       <c r="Z45" s="1"/>
-      <c r="AA45" s="1"/>
+      <c r="AA45" s="1">
+        <v>0</v>
+      </c>
       <c r="AB45" s="1">
         <v>0</v>
       </c>
@@ -3425,7 +3580,9 @@
       </c>
       <c r="Y46" s="1"/>
       <c r="Z46" s="1"/>
-      <c r="AA46" s="1"/>
+      <c r="AA46" s="1">
+        <v>0</v>
+      </c>
       <c r="AB46" s="1">
         <v>0</v>
       </c>
@@ -3466,7 +3623,9 @@
       </c>
       <c r="Y47" s="1"/>
       <c r="Z47" s="1"/>
-      <c r="AA47" s="1"/>
+      <c r="AA47" s="1">
+        <v>0</v>
+      </c>
       <c r="AB47" s="1">
         <v>0</v>
       </c>
@@ -3507,7 +3666,9 @@
       </c>
       <c r="Y48" s="1"/>
       <c r="Z48" s="1"/>
-      <c r="AA48" s="1"/>
+      <c r="AA48" s="1">
+        <v>0</v>
+      </c>
       <c r="AB48" s="1">
         <v>0</v>
       </c>
@@ -3549,7 +3710,9 @@
       <c r="X49" s="1"/>
       <c r="Y49" s="1"/>
       <c r="Z49" s="1"/>
-      <c r="AA49" s="1"/>
+      <c r="AA49" s="1">
+        <v>0</v>
+      </c>
       <c r="AB49" s="1">
         <v>0</v>
       </c>
@@ -3591,7 +3754,9 @@
       <c r="X50" s="1"/>
       <c r="Y50" s="1"/>
       <c r="Z50" s="1"/>
-      <c r="AA50" s="1"/>
+      <c r="AA50" s="1">
+        <v>0</v>
+      </c>
       <c r="AB50" s="1">
         <v>0</v>
       </c>
@@ -3633,7 +3798,9 @@
       <c r="X51" s="1"/>
       <c r="Y51" s="1"/>
       <c r="Z51" s="1"/>
-      <c r="AA51" s="1"/>
+      <c r="AA51" s="1">
+        <v>0</v>
+      </c>
       <c r="AB51" s="1">
         <v>0</v>
       </c>
@@ -3675,7 +3842,9 @@
       <c r="X52" s="1"/>
       <c r="Y52" s="1"/>
       <c r="Z52" s="1"/>
-      <c r="AA52" s="1"/>
+      <c r="AA52" s="1">
+        <v>0</v>
+      </c>
       <c r="AB52" s="1">
         <v>0</v>
       </c>
@@ -3717,7 +3886,9 @@
       <c r="X53" s="1"/>
       <c r="Y53" s="1"/>
       <c r="Z53" s="1"/>
-      <c r="AA53" s="1"/>
+      <c r="AA53" s="1">
+        <v>0</v>
+      </c>
       <c r="AB53" s="1">
         <v>0</v>
       </c>
@@ -3759,7 +3930,9 @@
       <c r="X54" s="1"/>
       <c r="Y54" s="1"/>
       <c r="Z54" s="1"/>
-      <c r="AA54" s="1"/>
+      <c r="AA54" s="1">
+        <v>0</v>
+      </c>
       <c r="AB54" s="1">
         <v>0</v>
       </c>
@@ -3802,7 +3975,9 @@
       <c r="X55" s="1"/>
       <c r="Y55" s="1"/>
       <c r="Z55" s="1"/>
-      <c r="AA55" s="1"/>
+      <c r="AA55" s="1">
+        <v>0</v>
+      </c>
       <c r="AB55" s="1">
         <v>0</v>
       </c>
@@ -3845,7 +4020,9 @@
       <c r="X56" s="1"/>
       <c r="Y56" s="1"/>
       <c r="Z56" s="1"/>
-      <c r="AA56" s="1"/>
+      <c r="AA56" s="1">
+        <v>0</v>
+      </c>
       <c r="AB56" s="1">
         <v>0</v>
       </c>
@@ -3888,7 +4065,9 @@
       <c r="X57" s="1"/>
       <c r="Y57" s="1"/>
       <c r="Z57" s="1"/>
-      <c r="AA57" s="1"/>
+      <c r="AA57" s="1">
+        <v>0</v>
+      </c>
       <c r="AB57" s="1">
         <v>0</v>
       </c>
@@ -3931,7 +4110,9 @@
       <c r="X58" s="1"/>
       <c r="Y58" s="1"/>
       <c r="Z58" s="1"/>
-      <c r="AA58" s="1"/>
+      <c r="AA58" s="1">
+        <v>0</v>
+      </c>
       <c r="AB58" s="1">
         <v>0</v>
       </c>
@@ -3974,7 +4155,9 @@
       <c r="X59" s="1"/>
       <c r="Y59" s="1"/>
       <c r="Z59" s="1"/>
-      <c r="AA59" s="1"/>
+      <c r="AA59" s="1">
+        <v>0</v>
+      </c>
       <c r="AB59" s="1">
         <v>0</v>
       </c>
@@ -4018,7 +4201,9 @@
       <c r="X60" s="1"/>
       <c r="Y60" s="1"/>
       <c r="Z60" s="1"/>
-      <c r="AA60" s="1"/>
+      <c r="AA60" s="1">
+        <v>0</v>
+      </c>
       <c r="AB60" s="1">
         <v>0</v>
       </c>
@@ -4062,7 +4247,9 @@
       <c r="X61" s="1"/>
       <c r="Y61" s="1"/>
       <c r="Z61" s="1"/>
-      <c r="AA61" s="1"/>
+      <c r="AA61" s="1">
+        <v>0</v>
+      </c>
       <c r="AB61" s="1">
         <v>0</v>
       </c>
@@ -4107,7 +4294,9 @@
       <c r="X62" s="1"/>
       <c r="Y62" s="1"/>
       <c r="Z62" s="1"/>
-      <c r="AA62" s="1"/>
+      <c r="AA62" s="1">
+        <v>0</v>
+      </c>
       <c r="AB62" s="1">
         <v>0</v>
       </c>
@@ -4152,7 +4341,9 @@
       <c r="X63" s="1"/>
       <c r="Y63" s="1"/>
       <c r="Z63" s="1"/>
-      <c r="AA63" s="1"/>
+      <c r="AA63" s="1">
+        <v>0</v>
+      </c>
       <c r="AB63" s="1">
         <v>0</v>
       </c>
@@ -4197,7 +4388,9 @@
       <c r="X64" s="1"/>
       <c r="Y64" s="1"/>
       <c r="Z64" s="1"/>
-      <c r="AA64" s="1"/>
+      <c r="AA64" s="1">
+        <v>0</v>
+      </c>
       <c r="AB64" s="1">
         <v>0</v>
       </c>
@@ -4242,7 +4435,9 @@
       <c r="X65" s="1"/>
       <c r="Y65" s="1"/>
       <c r="Z65" s="1"/>
-      <c r="AA65" s="1"/>
+      <c r="AA65" s="1">
+        <v>0</v>
+      </c>
       <c r="AB65" s="1">
         <v>0</v>
       </c>
@@ -4347,7 +4542,9 @@
       <c r="X67" s="1"/>
       <c r="Y67" s="1"/>
       <c r="Z67" s="1"/>
-      <c r="AA67" s="1"/>
+      <c r="AA67" s="1">
+        <v>0</v>
+      </c>
       <c r="AB67" s="1">
         <v>0</v>
       </c>
@@ -4393,7 +4590,9 @@
       <c r="X68" s="1"/>
       <c r="Y68" s="1"/>
       <c r="Z68" s="1"/>
-      <c r="AA68" s="1"/>
+      <c r="AA68" s="1">
+        <v>0</v>
+      </c>
       <c r="AB68" s="1">
         <v>0</v>
       </c>
@@ -4439,7 +4638,9 @@
       <c r="X69" s="1"/>
       <c r="Y69" s="1"/>
       <c r="Z69" s="1"/>
-      <c r="AA69" s="1"/>
+      <c r="AA69" s="1">
+        <v>0</v>
+      </c>
       <c r="AB69" s="1">
         <v>0</v>
       </c>
@@ -4485,7 +4686,9 @@
       <c r="X70" s="1"/>
       <c r="Y70" s="1"/>
       <c r="Z70" s="1"/>
-      <c r="AA70" s="1"/>
+      <c r="AA70" s="1">
+        <v>0</v>
+      </c>
       <c r="AB70" s="1">
         <v>0</v>
       </c>
@@ -4531,7 +4734,9 @@
       <c r="X71" s="1"/>
       <c r="Y71" s="1"/>
       <c r="Z71" s="1"/>
-      <c r="AA71" s="1"/>
+      <c r="AA71" s="1">
+        <v>0</v>
+      </c>
       <c r="AB71" s="1">
         <v>0</v>
       </c>
@@ -4578,7 +4783,9 @@
       <c r="X72" s="1"/>
       <c r="Y72" s="1"/>
       <c r="Z72" s="1"/>
-      <c r="AA72" s="1"/>
+      <c r="AA72" s="1">
+        <v>0</v>
+      </c>
       <c r="AB72" s="1">
         <v>0</v>
       </c>
@@ -4625,7 +4832,9 @@
       <c r="X73" s="1"/>
       <c r="Y73" s="1"/>
       <c r="Z73" s="1"/>
-      <c r="AA73" s="1"/>
+      <c r="AA73" s="1">
+        <v>0</v>
+      </c>
       <c r="AB73" s="1">
         <v>0</v>
       </c>
@@ -4672,7 +4881,9 @@
       <c r="X74" s="1"/>
       <c r="Y74" s="1"/>
       <c r="Z74" s="1"/>
-      <c r="AA74" s="1"/>
+      <c r="AA74" s="1">
+        <v>0</v>
+      </c>
       <c r="AB74" s="1">
         <v>0</v>
       </c>
@@ -4719,7 +4930,9 @@
       <c r="X75" s="1"/>
       <c r="Y75" s="1"/>
       <c r="Z75" s="1"/>
-      <c r="AA75" s="1"/>
+      <c r="AA75" s="1">
+        <v>0</v>
+      </c>
       <c r="AB75" s="1">
         <v>0</v>
       </c>
@@ -4766,7 +4979,9 @@
       <c r="X76" s="1"/>
       <c r="Y76" s="1"/>
       <c r="Z76" s="1"/>
-      <c r="AA76" s="1"/>
+      <c r="AA76" s="1">
+        <v>0</v>
+      </c>
       <c r="AB76" s="1">
         <v>0</v>
       </c>
@@ -4814,7 +5029,9 @@
       <c r="X77" s="1"/>
       <c r="Y77" s="1"/>
       <c r="Z77" s="1"/>
-      <c r="AA77" s="1"/>
+      <c r="AA77" s="1">
+        <v>0</v>
+      </c>
       <c r="AB77" s="1">
         <v>0</v>
       </c>
@@ -4862,7 +5079,9 @@
       <c r="X78" s="1"/>
       <c r="Y78" s="1"/>
       <c r="Z78" s="1"/>
-      <c r="AA78" s="1"/>
+      <c r="AA78" s="1">
+        <v>0</v>
+      </c>
       <c r="AB78" s="1">
         <v>0</v>
       </c>
@@ -4911,7 +5130,9 @@
       <c r="X79" s="1"/>
       <c r="Y79" s="1"/>
       <c r="Z79" s="1"/>
-      <c r="AA79" s="1"/>
+      <c r="AA79" s="1">
+        <v>0</v>
+      </c>
       <c r="AB79" s="1">
         <v>0</v>
       </c>
@@ -4960,7 +5181,9 @@
       <c r="X80" s="1"/>
       <c r="Y80" s="1"/>
       <c r="Z80" s="1"/>
-      <c r="AA80" s="1"/>
+      <c r="AA80" s="1">
+        <v>0</v>
+      </c>
       <c r="AB80" s="1">
         <v>0</v>
       </c>
@@ -5009,7 +5232,9 @@
       <c r="X81" s="1"/>
       <c r="Y81" s="1"/>
       <c r="Z81" s="1"/>
-      <c r="AA81" s="1"/>
+      <c r="AA81" s="1">
+        <v>0</v>
+      </c>
       <c r="AB81" s="1">
         <v>0</v>
       </c>
@@ -5058,7 +5283,9 @@
       <c r="X82" s="1"/>
       <c r="Y82" s="1"/>
       <c r="Z82" s="1"/>
-      <c r="AA82" s="1"/>
+      <c r="AA82" s="1">
+        <v>0</v>
+      </c>
       <c r="AB82" s="1">
         <v>0</v>
       </c>
@@ -5107,7 +5334,9 @@
       <c r="X83" s="1"/>
       <c r="Y83" s="1"/>
       <c r="Z83" s="1"/>
-      <c r="AA83" s="1"/>
+      <c r="AA83" s="1">
+        <v>0</v>
+      </c>
       <c r="AB83" s="1">
         <v>0</v>
       </c>
@@ -5157,7 +5386,9 @@
       <c r="X84" s="1"/>
       <c r="Y84" s="1"/>
       <c r="Z84" s="1"/>
-      <c r="AA84" s="1"/>
+      <c r="AA84" s="1">
+        <v>0</v>
+      </c>
       <c r="AB84" s="1">
         <v>0</v>
       </c>
@@ -5207,7 +5438,9 @@
       <c r="X85" s="1"/>
       <c r="Y85" s="1"/>
       <c r="Z85" s="1"/>
-      <c r="AA85" s="1"/>
+      <c r="AA85" s="1">
+        <v>0</v>
+      </c>
       <c r="AB85" s="1">
         <v>0</v>
       </c>
@@ -5257,7 +5490,9 @@
       <c r="X86" s="1"/>
       <c r="Y86" s="1"/>
       <c r="Z86" s="1"/>
-      <c r="AA86" s="1"/>
+      <c r="AA86" s="1">
+        <v>0</v>
+      </c>
       <c r="AB86" s="1">
         <v>0</v>
       </c>
@@ -5307,7 +5542,9 @@
       <c r="X87" s="1"/>
       <c r="Y87" s="1"/>
       <c r="Z87" s="1"/>
-      <c r="AA87" s="1"/>
+      <c r="AA87" s="1">
+        <v>0</v>
+      </c>
       <c r="AB87" s="1">
         <v>0</v>
       </c>
@@ -5358,7 +5595,9 @@
       <c r="X88" s="1"/>
       <c r="Y88" s="1"/>
       <c r="Z88" s="1"/>
-      <c r="AA88" s="1"/>
+      <c r="AA88" s="1">
+        <v>0</v>
+      </c>
       <c r="AB88" s="1">
         <v>0</v>
       </c>
@@ -5409,7 +5648,9 @@
       <c r="X89" s="1"/>
       <c r="Y89" s="1"/>
       <c r="Z89" s="1"/>
-      <c r="AA89" s="1"/>
+      <c r="AA89" s="1">
+        <v>0</v>
+      </c>
       <c r="AB89" s="1">
         <v>0</v>
       </c>
@@ -5460,7 +5701,9 @@
       <c r="X90" s="1"/>
       <c r="Y90" s="1"/>
       <c r="Z90" s="1"/>
-      <c r="AA90" s="1"/>
+      <c r="AA90" s="1">
+        <v>0</v>
+      </c>
       <c r="AB90" s="1">
         <v>0</v>
       </c>
@@ -5511,7 +5754,9 @@
       <c r="X91" s="1"/>
       <c r="Y91" s="1"/>
       <c r="Z91" s="1"/>
-      <c r="AA91" s="1"/>
+      <c r="AA91" s="1">
+        <v>0</v>
+      </c>
       <c r="AB91" s="1">
         <v>0</v>
       </c>
@@ -5562,7 +5807,9 @@
       <c r="X92" s="1"/>
       <c r="Y92" s="1"/>
       <c r="Z92" s="1"/>
-      <c r="AA92" s="1"/>
+      <c r="AA92" s="1">
+        <v>0</v>
+      </c>
       <c r="AB92" s="1">
         <v>0</v>
       </c>
@@ -5614,7 +5861,9 @@
       <c r="X93" s="1"/>
       <c r="Y93" s="1"/>
       <c r="Z93" s="1"/>
-      <c r="AA93" s="1"/>
+      <c r="AA93" s="1">
+        <v>0</v>
+      </c>
       <c r="AB93" s="1">
         <v>0</v>
       </c>
@@ -5666,7 +5915,9 @@
       <c r="X94" s="1"/>
       <c r="Y94" s="1"/>
       <c r="Z94" s="1"/>
-      <c r="AA94" s="1"/>
+      <c r="AA94" s="1">
+        <v>0</v>
+      </c>
       <c r="AB94" s="1">
         <v>0</v>
       </c>
@@ -5718,7 +5969,9 @@
       <c r="X95" s="1"/>
       <c r="Y95" s="1"/>
       <c r="Z95" s="1"/>
-      <c r="AA95" s="1"/>
+      <c r="AA95" s="1">
+        <v>0</v>
+      </c>
       <c r="AB95" s="1">
         <v>0</v>
       </c>
@@ -5770,7 +6023,9 @@
       <c r="X96" s="1"/>
       <c r="Y96" s="1"/>
       <c r="Z96" s="1"/>
-      <c r="AA96" s="1"/>
+      <c r="AA96" s="1">
+        <v>0</v>
+      </c>
       <c r="AB96" s="1">
         <v>0</v>
       </c>
@@ -5822,7 +6077,9 @@
       <c r="X97" s="1"/>
       <c r="Y97" s="1"/>
       <c r="Z97" s="1"/>
-      <c r="AA97" s="1"/>
+      <c r="AA97" s="1">
+        <v>0</v>
+      </c>
       <c r="AB97" s="1">
         <v>0</v>
       </c>
@@ -5875,7 +6132,9 @@
       <c r="X98" s="1"/>
       <c r="Y98" s="1"/>
       <c r="Z98" s="1"/>
-      <c r="AA98" s="1"/>
+      <c r="AA98" s="1">
+        <v>0</v>
+      </c>
       <c r="AB98" s="1">
         <v>0</v>
       </c>
@@ -5928,7 +6187,9 @@
       <c r="X99" s="1"/>
       <c r="Y99" s="1"/>
       <c r="Z99" s="1"/>
-      <c r="AA99" s="1"/>
+      <c r="AA99" s="1">
+        <v>0</v>
+      </c>
       <c r="AB99" s="1">
         <v>0</v>
       </c>
@@ -5981,7 +6242,9 @@
       <c r="X100" s="1"/>
       <c r="Y100" s="1"/>
       <c r="Z100" s="1"/>
-      <c r="AA100" s="1"/>
+      <c r="AA100" s="1">
+        <v>0</v>
+      </c>
       <c r="AB100" s="1">
         <v>0</v>
       </c>
@@ -6034,7 +6297,9 @@
       <c r="X101" s="1"/>
       <c r="Y101" s="1"/>
       <c r="Z101" s="1"/>
-      <c r="AA101" s="1"/>
+      <c r="AA101" s="1">
+        <v>0</v>
+      </c>
       <c r="AB101" s="1">
         <v>0</v>
       </c>
@@ -6088,7 +6353,9 @@
       <c r="X102" s="1"/>
       <c r="Y102" s="1"/>
       <c r="Z102" s="1"/>
-      <c r="AA102" s="1"/>
+      <c r="AA102" s="1">
+        <v>0</v>
+      </c>
       <c r="AB102" s="1">
         <v>0</v>
       </c>
@@ -6142,7 +6409,9 @@
       <c r="X103" s="1"/>
       <c r="Y103" s="1"/>
       <c r="Z103" s="1"/>
-      <c r="AA103" s="1"/>
+      <c r="AA103" s="1">
+        <v>0</v>
+      </c>
       <c r="AB103" s="1">
         <v>0</v>
       </c>
@@ -6197,7 +6466,9 @@
       <c r="X104" s="1"/>
       <c r="Y104" s="1"/>
       <c r="Z104" s="1"/>
-      <c r="AA104" s="1"/>
+      <c r="AA104" s="1">
+        <v>0</v>
+      </c>
       <c r="AB104" s="1">
         <v>0</v>
       </c>
@@ -6252,7 +6523,9 @@
       <c r="X105" s="1"/>
       <c r="Y105" s="1"/>
       <c r="Z105" s="1"/>
-      <c r="AA105" s="1"/>
+      <c r="AA105" s="1">
+        <v>0</v>
+      </c>
       <c r="AB105" s="1">
         <v>0</v>
       </c>
@@ -6307,7 +6580,9 @@
       <c r="X106" s="1"/>
       <c r="Y106" s="1"/>
       <c r="Z106" s="1"/>
-      <c r="AA106" s="1"/>
+      <c r="AA106" s="1">
+        <v>0</v>
+      </c>
       <c r="AB106" s="1">
         <v>0</v>
       </c>
@@ -6363,7 +6638,9 @@
       <c r="X107" s="1"/>
       <c r="Y107" s="1"/>
       <c r="Z107" s="1"/>
-      <c r="AA107" s="1"/>
+      <c r="AA107" s="1">
+        <v>0</v>
+      </c>
       <c r="AB107" s="1">
         <v>0</v>
       </c>
@@ -6419,7 +6696,9 @@
       <c r="X108" s="1"/>
       <c r="Y108" s="1"/>
       <c r="Z108" s="1"/>
-      <c r="AA108" s="1"/>
+      <c r="AA108" s="1">
+        <v>0</v>
+      </c>
       <c r="AB108" s="1">
         <v>0</v>
       </c>
@@ -6475,7 +6754,9 @@
       <c r="X109" s="1"/>
       <c r="Y109" s="1"/>
       <c r="Z109" s="1"/>
-      <c r="AA109" s="1"/>
+      <c r="AA109" s="1">
+        <v>0</v>
+      </c>
       <c r="AB109" s="1">
         <v>0</v>
       </c>
@@ -6532,7 +6813,9 @@
       <c r="X110" s="1"/>
       <c r="Y110" s="1"/>
       <c r="Z110" s="1"/>
-      <c r="AA110" s="1"/>
+      <c r="AA110" s="1">
+        <v>0</v>
+      </c>
       <c r="AB110" s="1">
         <v>0</v>
       </c>
@@ -6589,7 +6872,9 @@
       <c r="X111" s="1"/>
       <c r="Y111" s="1"/>
       <c r="Z111" s="1"/>
-      <c r="AA111" s="1"/>
+      <c r="AA111" s="1">
+        <v>0</v>
+      </c>
       <c r="AB111" s="1">
         <v>0</v>
       </c>
@@ -6646,7 +6931,9 @@
       <c r="X112" s="1"/>
       <c r="Y112" s="1"/>
       <c r="Z112" s="1"/>
-      <c r="AA112" s="1"/>
+      <c r="AA112" s="1">
+        <v>0</v>
+      </c>
       <c r="AB112" s="1">
         <v>0</v>
       </c>
@@ -6704,7 +6991,9 @@
       <c r="X113" s="1"/>
       <c r="Y113" s="1"/>
       <c r="Z113" s="1"/>
-      <c r="AA113" s="1"/>
+      <c r="AA113" s="1">
+        <v>0</v>
+      </c>
       <c r="AB113" s="1">
         <v>0</v>
       </c>
@@ -6762,7 +7051,9 @@
       <c r="X114" s="1"/>
       <c r="Y114" s="1"/>
       <c r="Z114" s="1"/>
-      <c r="AA114" s="1"/>
+      <c r="AA114" s="1">
+        <v>0</v>
+      </c>
       <c r="AB114" s="1">
         <v>0</v>
       </c>
@@ -6821,7 +7112,9 @@
       <c r="X115" s="1"/>
       <c r="Y115" s="1"/>
       <c r="Z115" s="1"/>
-      <c r="AA115" s="1"/>
+      <c r="AA115" s="1">
+        <v>0</v>
+      </c>
       <c r="AB115" s="1">
         <v>0</v>
       </c>
@@ -6880,7 +7173,9 @@
       <c r="X116" s="1"/>
       <c r="Y116" s="1"/>
       <c r="Z116" s="1"/>
-      <c r="AA116" s="1"/>
+      <c r="AA116" s="1">
+        <v>0</v>
+      </c>
       <c r="AB116" s="1">
         <v>0</v>
       </c>
@@ -6939,7 +7234,9 @@
       <c r="X117" s="1"/>
       <c r="Y117" s="1"/>
       <c r="Z117" s="1"/>
-      <c r="AA117" s="1"/>
+      <c r="AA117" s="1">
+        <v>0</v>
+      </c>
       <c r="AB117" s="1">
         <v>0</v>
       </c>
@@ -6999,7 +7296,9 @@
       <c r="X118" s="1"/>
       <c r="Y118" s="1"/>
       <c r="Z118" s="1"/>
-      <c r="AA118" s="1"/>
+      <c r="AA118" s="1">
+        <v>0</v>
+      </c>
       <c r="AB118" s="1">
         <v>0</v>
       </c>
@@ -7059,7 +7358,9 @@
       <c r="X119" s="1"/>
       <c r="Y119" s="1"/>
       <c r="Z119" s="1"/>
-      <c r="AA119" s="1"/>
+      <c r="AA119" s="1">
+        <v>0</v>
+      </c>
       <c r="AB119" s="1">
         <v>0</v>
       </c>
@@ -7119,7 +7420,9 @@
       <c r="X120" s="1"/>
       <c r="Y120" s="1"/>
       <c r="Z120" s="1"/>
-      <c r="AA120" s="1"/>
+      <c r="AA120" s="1">
+        <v>0</v>
+      </c>
       <c r="AB120" s="1">
         <v>0</v>
       </c>
@@ -7180,7 +7483,9 @@
       <c r="X121" s="1"/>
       <c r="Y121" s="1"/>
       <c r="Z121" s="1"/>
-      <c r="AA121" s="1"/>
+      <c r="AA121" s="1">
+        <v>0</v>
+      </c>
       <c r="AB121" s="1">
         <v>0</v>
       </c>
@@ -7241,7 +7546,9 @@
       <c r="X122" s="1"/>
       <c r="Y122" s="1"/>
       <c r="Z122" s="1"/>
-      <c r="AA122" s="1"/>
+      <c r="AA122" s="1">
+        <v>0</v>
+      </c>
       <c r="AB122" s="1">
         <v>0</v>
       </c>
@@ -7302,7 +7609,9 @@
       <c r="X123" s="1"/>
       <c r="Y123" s="1"/>
       <c r="Z123" s="1"/>
-      <c r="AA123" s="1"/>
+      <c r="AA123" s="1">
+        <v>0</v>
+      </c>
       <c r="AB123" s="1">
         <v>0</v>
       </c>
@@ -7364,7 +7673,9 @@
       <c r="X124" s="1"/>
       <c r="Y124" s="1"/>
       <c r="Z124" s="1"/>
-      <c r="AA124" s="1"/>
+      <c r="AA124" s="1">
+        <v>0</v>
+      </c>
       <c r="AB124" s="1">
         <v>0</v>
       </c>
@@ -10804,9 +11115,22 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="6.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -10874,7 +11198,58 @@
       </c>
       <c r="B2">
         <f>SUM(C2:C2:S2)</f>
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2">
+        <v>1</v>
+      </c>
+      <c r="O2">
+        <v>1</v>
+      </c>
+      <c r="P2">
+        <v>1</v>
+      </c>
+      <c r="Q2">
+        <v>1</v>
+      </c>
+      <c r="R2">
+        <v>1</v>
+      </c>
+      <c r="S2">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
@@ -10883,7 +11258,58 @@
       </c>
       <c r="B3">
         <f>SUM(C3:C3:S3)</f>
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>1</v>
+      </c>
+      <c r="O3">
+        <v>1</v>
+      </c>
+      <c r="P3">
+        <v>1</v>
+      </c>
+      <c r="Q3">
+        <v>1</v>
+      </c>
+      <c r="R3">
+        <v>1</v>
+      </c>
+      <c r="S3">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
@@ -10892,7 +11318,58 @@
       </c>
       <c r="B4">
         <f>SUM(C4:C4:S4)</f>
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+      <c r="N4">
+        <v>1</v>
+      </c>
+      <c r="O4">
+        <v>1</v>
+      </c>
+      <c r="P4">
+        <v>1</v>
+      </c>
+      <c r="Q4">
+        <v>1</v>
+      </c>
+      <c r="R4">
+        <v>1</v>
+      </c>
+      <c r="S4">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -10901,7 +11378,58 @@
       </c>
       <c r="B5">
         <f>SUM(C5:C5:S5)</f>
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+      <c r="N5">
+        <v>1</v>
+      </c>
+      <c r="O5">
+        <v>1</v>
+      </c>
+      <c r="P5">
+        <v>1</v>
+      </c>
+      <c r="Q5">
+        <v>1</v>
+      </c>
+      <c r="R5">
+        <v>1</v>
+      </c>
+      <c r="S5">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
@@ -10910,7 +11438,58 @@
       </c>
       <c r="B6">
         <f>SUM(C6:C6:S6)</f>
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+      <c r="N6">
+        <v>1</v>
+      </c>
+      <c r="O6">
+        <v>1</v>
+      </c>
+      <c r="P6">
+        <v>1</v>
+      </c>
+      <c r="Q6">
+        <v>1</v>
+      </c>
+      <c r="R6">
+        <v>1</v>
+      </c>
+      <c r="S6">
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
@@ -10919,7 +11498,58 @@
       </c>
       <c r="B7">
         <f>SUM(C7:C7:S7)</f>
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
+      <c r="N7">
+        <v>1</v>
+      </c>
+      <c r="O7">
+        <v>1</v>
+      </c>
+      <c r="P7">
+        <v>1</v>
+      </c>
+      <c r="Q7">
+        <v>1</v>
+      </c>
+      <c r="R7">
+        <v>1</v>
+      </c>
+      <c r="S7">
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
@@ -10928,7 +11558,58 @@
       </c>
       <c r="B8">
         <f>SUM(C8:C8:S8)</f>
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8">
+        <v>1</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8">
+        <v>1</v>
+      </c>
+      <c r="N8">
+        <v>1</v>
+      </c>
+      <c r="O8">
+        <v>1</v>
+      </c>
+      <c r="P8">
+        <v>1</v>
+      </c>
+      <c r="Q8">
+        <v>1</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8">
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
@@ -10937,7 +11618,58 @@
       </c>
       <c r="B9">
         <f>SUM(C9:C9:S9)</f>
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9">
+        <v>1</v>
+      </c>
+      <c r="N9">
+        <v>1</v>
+      </c>
+      <c r="O9">
+        <v>1</v>
+      </c>
+      <c r="P9">
+        <v>1</v>
+      </c>
+      <c r="Q9">
+        <v>1</v>
+      </c>
+      <c r="R9">
+        <v>1</v>
+      </c>
+      <c r="S9">
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
@@ -10946,7 +11678,58 @@
       </c>
       <c r="B10">
         <f>SUM(C10:C10:S10)</f>
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10">
+        <v>1</v>
+      </c>
+      <c r="N10">
+        <v>1</v>
+      </c>
+      <c r="O10">
+        <v>1</v>
+      </c>
+      <c r="P10">
+        <v>1</v>
+      </c>
+      <c r="Q10">
+        <v>1</v>
+      </c>
+      <c r="R10">
+        <v>1</v>
+      </c>
+      <c r="S10">
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
@@ -10955,7 +11738,58 @@
       </c>
       <c r="B11">
         <f>SUM(C11:C11:S11)</f>
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11">
+        <v>1</v>
+      </c>
+      <c r="N11">
+        <v>1</v>
+      </c>
+      <c r="O11">
+        <v>1</v>
+      </c>
+      <c r="P11">
+        <v>1</v>
+      </c>
+      <c r="Q11">
+        <v>1</v>
+      </c>
+      <c r="R11">
+        <v>1</v>
+      </c>
+      <c r="S11">
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
@@ -10964,7 +11798,58 @@
       </c>
       <c r="B12">
         <f>SUM(C12:C12:S12)</f>
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <v>1</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
+      <c r="K12">
+        <v>1</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12">
+        <v>1</v>
+      </c>
+      <c r="N12">
+        <v>1</v>
+      </c>
+      <c r="O12">
+        <v>1</v>
+      </c>
+      <c r="P12">
+        <v>1</v>
+      </c>
+      <c r="Q12">
+        <v>1</v>
+      </c>
+      <c r="R12">
+        <v>1</v>
+      </c>
+      <c r="S12">
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
@@ -10973,7 +11858,58 @@
       </c>
       <c r="B13">
         <f>SUM(C13:C13:S13)</f>
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>1</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="J13">
+        <v>1</v>
+      </c>
+      <c r="K13">
+        <v>1</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13">
+        <v>1</v>
+      </c>
+      <c r="N13">
+        <v>1</v>
+      </c>
+      <c r="O13">
+        <v>1</v>
+      </c>
+      <c r="P13">
+        <v>1</v>
+      </c>
+      <c r="Q13">
+        <v>1</v>
+      </c>
+      <c r="R13">
+        <v>1</v>
+      </c>
+      <c r="S13">
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
@@ -10982,7 +11918,58 @@
       </c>
       <c r="B14">
         <f>SUM(C14:C14:S14)</f>
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <v>1</v>
+      </c>
+      <c r="J14">
+        <v>1</v>
+      </c>
+      <c r="K14">
+        <v>1</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14">
+        <v>1</v>
+      </c>
+      <c r="N14">
+        <v>1</v>
+      </c>
+      <c r="O14">
+        <v>1</v>
+      </c>
+      <c r="P14">
+        <v>1</v>
+      </c>
+      <c r="Q14">
+        <v>1</v>
+      </c>
+      <c r="R14">
+        <v>1</v>
+      </c>
+      <c r="S14">
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
@@ -10991,7 +11978,58 @@
       </c>
       <c r="B15">
         <f>SUM(C15:C15:S15)</f>
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
+      <c r="K15">
+        <v>1</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
+        <v>1</v>
+      </c>
+      <c r="O15">
+        <v>1</v>
+      </c>
+      <c r="P15">
+        <v>1</v>
+      </c>
+      <c r="Q15">
+        <v>1</v>
+      </c>
+      <c r="R15">
+        <v>1</v>
+      </c>
+      <c r="S15">
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
@@ -11000,78 +12038,537 @@
       </c>
       <c r="B16">
         <f>SUM(C16:C16:S16)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16">
+        <v>1</v>
+      </c>
+      <c r="J16">
+        <v>1</v>
+      </c>
+      <c r="K16">
+        <v>1</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16">
+        <v>1</v>
+      </c>
+      <c r="N16">
+        <v>1</v>
+      </c>
+      <c r="O16">
+        <v>1</v>
+      </c>
+      <c r="P16">
+        <v>1</v>
+      </c>
+      <c r="Q16">
+        <v>1</v>
+      </c>
+      <c r="R16">
+        <v>1</v>
+      </c>
+      <c r="S16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>16</v>
       </c>
       <c r="B17">
         <f>SUM(C17:C17:S17)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>1</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+      <c r="J17">
+        <v>1</v>
+      </c>
+      <c r="K17">
+        <v>1</v>
+      </c>
+      <c r="L17">
+        <v>1</v>
+      </c>
+      <c r="M17">
+        <v>1</v>
+      </c>
+      <c r="N17">
+        <v>1</v>
+      </c>
+      <c r="O17">
+        <v>1</v>
+      </c>
+      <c r="P17">
+        <v>1</v>
+      </c>
+      <c r="Q17">
+        <v>1</v>
+      </c>
+      <c r="R17">
+        <v>1</v>
+      </c>
+      <c r="S17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
       </c>
       <c r="B18">
         <f>SUM(C18:C18:S18)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>1</v>
+      </c>
+      <c r="I18">
+        <v>1</v>
+      </c>
+      <c r="J18">
+        <v>1</v>
+      </c>
+      <c r="K18">
+        <v>1</v>
+      </c>
+      <c r="L18">
+        <v>1</v>
+      </c>
+      <c r="M18">
+        <v>1</v>
+      </c>
+      <c r="N18">
+        <v>1</v>
+      </c>
+      <c r="O18">
+        <v>1</v>
+      </c>
+      <c r="P18">
+        <v>1</v>
+      </c>
+      <c r="Q18">
+        <v>1</v>
+      </c>
+      <c r="R18">
+        <v>1</v>
+      </c>
+      <c r="S18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>52</v>
       </c>
       <c r="B19">
         <f>SUM(C19:C19:S19)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>1</v>
+      </c>
+      <c r="P19">
+        <v>1</v>
+      </c>
+      <c r="Q19">
+        <v>0</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>18</v>
       </c>
       <c r="B20">
         <f>SUM(C20:C20:S20)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
+      </c>
+      <c r="I20">
+        <v>1</v>
+      </c>
+      <c r="J20">
+        <v>1</v>
+      </c>
+      <c r="K20">
+        <v>1</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
+      </c>
+      <c r="M20">
+        <v>1</v>
+      </c>
+      <c r="N20">
+        <v>0</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
+        <v>1</v>
+      </c>
+      <c r="R20">
+        <v>1</v>
+      </c>
+      <c r="S20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>19</v>
       </c>
       <c r="B21">
         <f>SUM(C21:C21:S21)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
+        <v>1</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
+        <v>1</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
+      <c r="J21">
+        <v>1</v>
+      </c>
+      <c r="K21">
+        <v>1</v>
+      </c>
+      <c r="L21">
+        <v>1</v>
+      </c>
+      <c r="M21">
+        <v>0</v>
+      </c>
+      <c r="N21">
+        <v>1</v>
+      </c>
+      <c r="O21">
+        <v>0</v>
+      </c>
+      <c r="P21">
+        <v>0</v>
+      </c>
+      <c r="Q21">
+        <v>0</v>
+      </c>
+      <c r="R21">
+        <v>0</v>
+      </c>
+      <c r="S21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>20</v>
       </c>
       <c r="B22">
         <f>SUM(C22:C22:S22)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22">
+        <v>1</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>1</v>
+      </c>
+      <c r="I22">
+        <v>1</v>
+      </c>
+      <c r="J22">
+        <v>1</v>
+      </c>
+      <c r="K22">
+        <v>1</v>
+      </c>
+      <c r="L22">
+        <v>1</v>
+      </c>
+      <c r="M22">
+        <v>0</v>
+      </c>
+      <c r="N22">
+        <v>1</v>
+      </c>
+      <c r="O22">
+        <v>0</v>
+      </c>
+      <c r="P22">
+        <v>0</v>
+      </c>
+      <c r="Q22">
+        <v>0</v>
+      </c>
+      <c r="R22">
+        <v>1</v>
+      </c>
+      <c r="S22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>21</v>
       </c>
       <c r="B23">
         <f>SUM(C23:C23:S23)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <v>1</v>
+      </c>
+      <c r="I23">
+        <v>1</v>
+      </c>
+      <c r="J23">
+        <v>1</v>
+      </c>
+      <c r="K23">
+        <v>1</v>
+      </c>
+      <c r="L23">
+        <v>1</v>
+      </c>
+      <c r="M23">
+        <v>1</v>
+      </c>
+      <c r="N23">
+        <v>1</v>
+      </c>
+      <c r="O23">
+        <v>1</v>
+      </c>
+      <c r="P23">
+        <v>1</v>
+      </c>
+      <c r="Q23">
+        <v>1</v>
+      </c>
+      <c r="R23">
+        <v>1</v>
+      </c>
+      <c r="S23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>22</v>
       </c>
       <c r="B24">
         <f>SUM(C24:C24:S24)</f>
+        <v>16</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+      <c r="H24">
+        <v>1</v>
+      </c>
+      <c r="I24">
+        <v>1</v>
+      </c>
+      <c r="J24">
+        <v>1</v>
+      </c>
+      <c r="K24">
+        <v>1</v>
+      </c>
+      <c r="L24">
+        <v>1</v>
+      </c>
+      <c r="M24">
+        <v>1</v>
+      </c>
+      <c r="N24">
+        <v>1</v>
+      </c>
+      <c r="O24">
+        <v>1</v>
+      </c>
+      <c r="P24">
+        <v>1</v>
+      </c>
+      <c r="Q24">
+        <v>1</v>
+      </c>
+      <c r="R24">
+        <v>1</v>
+      </c>
+      <c r="S24">
         <v>0</v>
       </c>
     </row>
@@ -11082,139 +12579,1450 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5D4303C-7F1D-4CBD-BF56-16C815E789BE}">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" t="s">
+        <v>32</v>
+      </c>
+      <c r="L1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M1" t="s">
+        <v>33</v>
+      </c>
+      <c r="N1" t="s">
+        <v>35</v>
+      </c>
+      <c r="O1" t="s">
+        <v>36</v>
+      </c>
+      <c r="P1" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>39</v>
+      </c>
+      <c r="R1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B2">
+        <f>SUM(C2:R2)</f>
+        <v>16</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2">
+        <v>1</v>
+      </c>
+      <c r="O2">
+        <v>1</v>
+      </c>
+      <c r="P2">
+        <v>1</v>
+      </c>
+      <c r="Q2">
+        <v>1</v>
+      </c>
+      <c r="R2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <f t="shared" ref="B3:B25" si="0">SUM(C3:R3)</f>
+        <v>16</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+      <c r="N3">
+        <v>1</v>
+      </c>
+      <c r="O3">
+        <v>1</v>
+      </c>
+      <c r="P3">
+        <v>1</v>
+      </c>
+      <c r="Q3">
+        <v>1</v>
+      </c>
+      <c r="R3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+      <c r="N4">
+        <v>1</v>
+      </c>
+      <c r="O4">
+        <v>1</v>
+      </c>
+      <c r="P4">
+        <v>1</v>
+      </c>
+      <c r="Q4">
+        <v>1</v>
+      </c>
+      <c r="R4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B5">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+      <c r="N5">
+        <v>1</v>
+      </c>
+      <c r="O5">
+        <v>1</v>
+      </c>
+      <c r="P5">
+        <v>1</v>
+      </c>
+      <c r="Q5">
+        <v>1</v>
+      </c>
+      <c r="R5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+      <c r="N6">
+        <v>1</v>
+      </c>
+      <c r="O6">
+        <v>1</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>1</v>
+      </c>
+      <c r="R6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
+      <c r="N7">
+        <v>1</v>
+      </c>
+      <c r="O7">
+        <v>1</v>
+      </c>
+      <c r="P7">
+        <v>1</v>
+      </c>
+      <c r="Q7">
+        <v>1</v>
+      </c>
+      <c r="R7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8">
+        <v>1</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8">
+        <v>1</v>
+      </c>
+      <c r="N8">
+        <v>1</v>
+      </c>
+      <c r="O8">
+        <v>1</v>
+      </c>
+      <c r="P8">
+        <v>1</v>
+      </c>
+      <c r="Q8">
+        <v>1</v>
+      </c>
+      <c r="R8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B9">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9">
+        <v>1</v>
+      </c>
+      <c r="N9">
+        <v>1</v>
+      </c>
+      <c r="O9">
+        <v>1</v>
+      </c>
+      <c r="P9">
+        <v>1</v>
+      </c>
+      <c r="Q9">
+        <v>1</v>
+      </c>
+      <c r="R9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B10">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10">
+        <v>1</v>
+      </c>
+      <c r="N10">
+        <v>1</v>
+      </c>
+      <c r="O10">
+        <v>1</v>
+      </c>
+      <c r="P10">
+        <v>1</v>
+      </c>
+      <c r="Q10">
+        <v>1</v>
+      </c>
+      <c r="R10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11">
+        <v>1</v>
+      </c>
+      <c r="N11">
+        <v>1</v>
+      </c>
+      <c r="O11">
+        <v>1</v>
+      </c>
+      <c r="P11">
+        <v>1</v>
+      </c>
+      <c r="Q11">
+        <v>1</v>
+      </c>
+      <c r="R11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
+      <c r="K12">
+        <v>1</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12">
+        <v>1</v>
+      </c>
+      <c r="N12">
+        <v>1</v>
+      </c>
+      <c r="O12">
+        <v>1</v>
+      </c>
+      <c r="P12">
+        <v>1</v>
+      </c>
+      <c r="Q12">
+        <v>1</v>
+      </c>
+      <c r="R12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>1</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="J13">
+        <v>1</v>
+      </c>
+      <c r="K13">
+        <v>1</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13">
+        <v>1</v>
+      </c>
+      <c r="N13">
+        <v>1</v>
+      </c>
+      <c r="O13">
+        <v>1</v>
+      </c>
+      <c r="P13">
+        <v>1</v>
+      </c>
+      <c r="Q13">
+        <v>1</v>
+      </c>
+      <c r="R13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B14">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <v>1</v>
+      </c>
+      <c r="J14">
+        <v>1</v>
+      </c>
+      <c r="K14">
+        <v>1</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14">
+        <v>1</v>
+      </c>
+      <c r="N14">
+        <v>1</v>
+      </c>
+      <c r="O14">
+        <v>1</v>
+      </c>
+      <c r="P14">
+        <v>1</v>
+      </c>
+      <c r="Q14">
+        <v>1</v>
+      </c>
+      <c r="R14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B15">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
+      <c r="K15">
+        <v>1</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15">
+        <v>1</v>
+      </c>
+      <c r="N15">
+        <v>1</v>
+      </c>
+      <c r="O15">
+        <v>1</v>
+      </c>
+      <c r="P15">
+        <v>1</v>
+      </c>
+      <c r="Q15">
+        <v>1</v>
+      </c>
+      <c r="R15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B16">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16">
+        <v>1</v>
+      </c>
+      <c r="J16">
+        <v>1</v>
+      </c>
+      <c r="K16">
+        <v>1</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16">
+        <v>1</v>
+      </c>
+      <c r="N16">
+        <v>1</v>
+      </c>
+      <c r="O16">
+        <v>1</v>
+      </c>
+      <c r="P16">
+        <v>1</v>
+      </c>
+      <c r="Q16">
+        <v>1</v>
+      </c>
+      <c r="R16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B17">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>1</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+      <c r="J17">
+        <v>1</v>
+      </c>
+      <c r="K17">
+        <v>1</v>
+      </c>
+      <c r="L17">
+        <v>1</v>
+      </c>
+      <c r="M17">
+        <v>1</v>
+      </c>
+      <c r="N17">
+        <v>1</v>
+      </c>
+      <c r="O17">
+        <v>1</v>
+      </c>
+      <c r="P17">
+        <v>1</v>
+      </c>
+      <c r="Q17">
+        <v>1</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B18">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18">
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="P18">
+        <v>1</v>
+      </c>
+      <c r="Q18">
+        <v>0</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B19">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19">
+        <v>0</v>
+      </c>
+      <c r="R19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
+      </c>
+      <c r="I20">
+        <v>1</v>
+      </c>
+      <c r="J20">
+        <v>1</v>
+      </c>
+      <c r="K20">
+        <v>1</v>
+      </c>
+      <c r="L20">
+        <v>1</v>
+      </c>
+      <c r="M20">
+        <v>1</v>
+      </c>
+      <c r="N20">
+        <v>1</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
+        <v>1</v>
+      </c>
+      <c r="R20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B21">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
+        <v>1</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
+        <v>1</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
+      <c r="J21">
+        <v>1</v>
+      </c>
+      <c r="K21">
+        <v>1</v>
+      </c>
+      <c r="L21">
+        <v>1</v>
+      </c>
+      <c r="M21">
+        <v>1</v>
+      </c>
+      <c r="N21">
+        <v>1</v>
+      </c>
+      <c r="O21">
+        <v>1</v>
+      </c>
+      <c r="P21">
+        <v>1</v>
+      </c>
+      <c r="Q21">
+        <v>1</v>
+      </c>
+      <c r="R21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B22">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22">
+        <v>1</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>1</v>
+      </c>
+      <c r="I22">
+        <v>1</v>
+      </c>
+      <c r="J22">
+        <v>1</v>
+      </c>
+      <c r="K22">
+        <v>1</v>
+      </c>
+      <c r="L22">
+        <v>1</v>
+      </c>
+      <c r="M22">
+        <v>1</v>
+      </c>
+      <c r="N22">
+        <v>0</v>
+      </c>
+      <c r="O22">
+        <v>0</v>
+      </c>
+      <c r="P22">
+        <v>0</v>
+      </c>
+      <c r="Q22">
+        <v>0</v>
+      </c>
+      <c r="R22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B23">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <v>1</v>
+      </c>
+      <c r="I23">
+        <v>1</v>
+      </c>
+      <c r="J23">
+        <v>1</v>
+      </c>
+      <c r="K23">
+        <v>1</v>
+      </c>
+      <c r="L23">
+        <v>1</v>
+      </c>
+      <c r="M23">
+        <v>1</v>
+      </c>
+      <c r="N23">
+        <v>1</v>
+      </c>
+      <c r="O23">
+        <v>1</v>
+      </c>
+      <c r="P23">
+        <v>1</v>
+      </c>
+      <c r="Q23">
+        <v>1</v>
+      </c>
+      <c r="R23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B24">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24">
+        <v>0</v>
+      </c>
+      <c r="N24">
+        <v>1</v>
+      </c>
+      <c r="O24">
+        <v>1</v>
+      </c>
+      <c r="P24">
+        <v>1</v>
+      </c>
+      <c r="Q24">
+        <v>1</v>
+      </c>
+      <c r="R24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>61</v>
+      </c>
+      <c r="B25">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25">
+        <v>0</v>
+      </c>
+      <c r="N25">
+        <v>0</v>
+      </c>
+      <c r="O25">
+        <v>1</v>
+      </c>
+      <c r="P25">
+        <v>1</v>
+      </c>
+      <c r="Q25">
+        <v>0</v>
+      </c>
+      <c r="R25">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>